<commit_message>
feat: Implement a robust evaluation script)
</commit_message>
<xml_diff>
--- a/Eval_Run_Logs.xlsx
+++ b/Eval_Run_Logs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\DeepRL-MsPacman\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D4C6BAD-DD81-4850-A49E-E3A95191803F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A01C34EB-9AB2-4A38-A3D1-832E0371793A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0D67D52D-1513-48BB-A273-B9082DA3F499}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{0D67D52D-1513-48BB-A273-B9082DA3F499}"/>
   </bookViews>
   <sheets>
     <sheet name="DQN_Runs" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="51">
   <si>
     <t>Run ID</t>
   </si>
@@ -129,9 +129,6 @@
     <t>dqn_1753323569</t>
   </si>
   <si>
-    <t>DQN Baseline - 10M steps - Default</t>
-  </si>
-  <si>
     <t>ppo_1753323765</t>
   </si>
   <si>
@@ -141,13 +138,58 @@
     <t>PPO Baseline - 10M steps</t>
   </si>
   <si>
-    <t>dqn_1753367403</t>
-  </si>
-  <si>
-    <t>DQN Baseline - 10M steps - High timestep penalty</t>
-  </si>
-  <si>
     <t>ppo_1753366805</t>
+  </si>
+  <si>
+    <t>PPO Baseline - 10M steps - Low LR</t>
+  </si>
+  <si>
+    <t>DQN Baseline - 10M steps - High Epsilon Decay Duration</t>
+  </si>
+  <si>
+    <t>DQN Baseline - 10M steps - Baseline</t>
+  </si>
+  <si>
+    <t>PPO Baseline - 10M steps - High LR</t>
+  </si>
+  <si>
+    <t>dqn_1753409992</t>
+  </si>
+  <si>
+    <t>DQN Baseline - 10M steps - Low LR</t>
+  </si>
+  <si>
+    <t>ppo_1753667491</t>
+  </si>
+  <si>
+    <t>dqn_1753667511</t>
+  </si>
+  <si>
+    <t>DQN Baseline - 10M steps - High LR</t>
+  </si>
+  <si>
+    <t>PPO Baseline - 10M steps - Low Epochs</t>
+  </si>
+  <si>
+    <t>PPO Baseline - 10M steps - High Epochs</t>
+  </si>
+  <si>
+    <t>DQN Baseline - 10M steps - Low Epsilon Decay Duration</t>
+  </si>
+  <si>
+    <t>DQN Baseline - 10M steps - Low Update Frequency</t>
+  </si>
+  <si>
+    <t>PPO Baseline - 10M steps - Medium n_steps</t>
+  </si>
+  <si>
+    <t>ppo_1753410334</t>
+  </si>
+  <si>
+    <t>DQN Baseline - 10M steps - High Update Frequency</t>
+  </si>
+  <si>
+    <t>PPO Baseline - 10M steps - High n_steps</t>
   </si>
 </sst>
 </file>
@@ -534,7 +576,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BDCA7AB-C83E-496B-A323-D25B7B27B0B8}">
-  <dimension ref="A1:V4"/>
+  <dimension ref="A1:V9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
@@ -640,7 +682,7 @@
         <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E2" s="1">
         <v>10000000</v>
@@ -652,7 +694,7 @@
         <v>250000</v>
       </c>
       <c r="H2" s="1">
-        <v>1000000</v>
+        <v>2500000</v>
       </c>
       <c r="I2" s="1">
         <v>10000</v>
@@ -684,7 +726,7 @@
         <v>45861</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s">
         <v>29</v>
@@ -699,7 +741,7 @@
         <v>250000</v>
       </c>
       <c r="H3" s="1">
-        <v>1000000</v>
+        <v>2500000</v>
       </c>
       <c r="I3" s="1">
         <v>10000</v>
@@ -731,10 +773,10 @@
         <v>45862</v>
       </c>
       <c r="C4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D4" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="E4" s="1">
         <v>10000000</v>
@@ -752,22 +794,245 @@
         <v>10000</v>
       </c>
       <c r="J4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4">
-        <v>-250</v>
+        <v>0</v>
       </c>
       <c r="L4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M4">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="N4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O4">
-        <v>-10</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <v>45865</v>
+      </c>
+      <c r="C5" t="s">
+        <v>39</v>
+      </c>
+      <c r="D5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E5" s="1">
+        <v>10000000</v>
+      </c>
+      <c r="F5">
+        <v>5.0000000000000002E-5</v>
+      </c>
+      <c r="G5" s="1">
+        <v>250000</v>
+      </c>
+      <c r="H5" s="1">
+        <v>1000000</v>
+      </c>
+      <c r="I5" s="1">
+        <v>10000</v>
+      </c>
+      <c r="J5" t="b">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5" t="b">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5" t="b">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <v>45866</v>
+      </c>
+      <c r="C6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E6" s="1">
+        <v>10000000</v>
+      </c>
+      <c r="F6">
+        <v>2.5000000000000001E-4</v>
+      </c>
+      <c r="G6" s="1">
+        <v>250000</v>
+      </c>
+      <c r="H6" s="1">
+        <v>1000000</v>
+      </c>
+      <c r="I6" s="1">
+        <v>10000</v>
+      </c>
+      <c r="J6" t="b">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6" t="b">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6" t="b">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <v>45861</v>
+      </c>
+      <c r="C7" t="s">
+        <v>45</v>
+      </c>
+      <c r="E7" s="1">
+        <v>10000000</v>
+      </c>
+      <c r="F7">
+        <v>1E-4</v>
+      </c>
+      <c r="G7" s="1">
+        <v>250000</v>
+      </c>
+      <c r="H7" s="1">
+        <v>500000</v>
+      </c>
+      <c r="I7" s="1">
+        <v>10000</v>
+      </c>
+      <c r="J7" t="b">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7" t="b">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2">
+        <v>45861</v>
+      </c>
+      <c r="C8" t="s">
+        <v>46</v>
+      </c>
+      <c r="E8" s="1">
+        <v>10000000</v>
+      </c>
+      <c r="F8">
+        <v>1E-4</v>
+      </c>
+      <c r="G8" s="1">
+        <v>250000</v>
+      </c>
+      <c r="H8" s="1">
+        <v>1000000</v>
+      </c>
+      <c r="I8" s="1">
+        <v>1000</v>
+      </c>
+      <c r="J8" t="b">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8" t="b">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8" t="b">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2">
+        <v>45861</v>
+      </c>
+      <c r="C9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" s="1">
+        <v>10000000</v>
+      </c>
+      <c r="F9">
+        <v>1E-4</v>
+      </c>
+      <c r="G9" s="1">
+        <v>250000</v>
+      </c>
+      <c r="H9" s="1">
+        <v>1000000</v>
+      </c>
+      <c r="I9" s="1">
+        <v>20000</v>
+      </c>
+      <c r="J9" t="b">
+        <v>0</v>
+      </c>
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9" t="b">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="N9" t="b">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -777,7 +1042,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{606356CF-33ED-426F-8480-D5D1647FF48E}">
-  <dimension ref="A1:X3"/>
+  <dimension ref="A1:X9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
@@ -888,10 +1153,10 @@
         <v>45861</v>
       </c>
       <c r="C2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E2" s="1">
         <v>10000000</v>
@@ -944,7 +1209,7 @@
         <v>28</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E3" s="1">
         <v>10000000</v>
@@ -984,6 +1249,312 @@
       </c>
       <c r="Q3">
         <v>-1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2">
+        <v>45862</v>
+      </c>
+      <c r="C4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D4" t="s">
+        <v>48</v>
+      </c>
+      <c r="E4" s="1">
+        <v>10000000</v>
+      </c>
+      <c r="F4">
+        <v>1E-4</v>
+      </c>
+      <c r="G4">
+        <v>128</v>
+      </c>
+      <c r="H4">
+        <v>4</v>
+      </c>
+      <c r="I4">
+        <v>0.1</v>
+      </c>
+      <c r="J4">
+        <v>0.01</v>
+      </c>
+      <c r="K4">
+        <v>0.95</v>
+      </c>
+      <c r="L4" t="b">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4" t="b">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <v>45865</v>
+      </c>
+      <c r="C5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" s="1">
+        <v>10000000</v>
+      </c>
+      <c r="F5">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G5">
+        <v>128</v>
+      </c>
+      <c r="H5">
+        <v>4</v>
+      </c>
+      <c r="I5">
+        <v>0.1</v>
+      </c>
+      <c r="J5">
+        <v>0.01</v>
+      </c>
+      <c r="K5">
+        <v>0.95</v>
+      </c>
+      <c r="L5" t="b">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5" t="b">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2">
+        <v>45866</v>
+      </c>
+      <c r="C6" t="s">
+        <v>43</v>
+      </c>
+      <c r="E6" s="1">
+        <v>10000000</v>
+      </c>
+      <c r="F6">
+        <v>2.5000000000000001E-4</v>
+      </c>
+      <c r="G6">
+        <v>128</v>
+      </c>
+      <c r="H6">
+        <v>3</v>
+      </c>
+      <c r="I6">
+        <v>0.1</v>
+      </c>
+      <c r="J6">
+        <v>0.01</v>
+      </c>
+      <c r="K6">
+        <v>0.95</v>
+      </c>
+      <c r="L6" t="b">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6" t="b">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2">
+        <v>45867</v>
+      </c>
+      <c r="C7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" s="1">
+        <v>10000000</v>
+      </c>
+      <c r="F7">
+        <v>2.5000000000000001E-4</v>
+      </c>
+      <c r="G7">
+        <v>128</v>
+      </c>
+      <c r="H7">
+        <v>10</v>
+      </c>
+      <c r="I7">
+        <v>0.1</v>
+      </c>
+      <c r="J7">
+        <v>0.01</v>
+      </c>
+      <c r="K7">
+        <v>0.95</v>
+      </c>
+      <c r="L7" t="b">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7" t="b">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>0</v>
+      </c>
+      <c r="P7" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2">
+        <v>45868</v>
+      </c>
+      <c r="C8" t="s">
+        <v>47</v>
+      </c>
+      <c r="E8" s="1">
+        <v>10000000</v>
+      </c>
+      <c r="F8">
+        <v>2.5000000000000001E-4</v>
+      </c>
+      <c r="G8">
+        <v>512</v>
+      </c>
+      <c r="H8">
+        <v>4</v>
+      </c>
+      <c r="I8">
+        <v>0.1</v>
+      </c>
+      <c r="J8">
+        <v>0.01</v>
+      </c>
+      <c r="K8">
+        <v>0.95</v>
+      </c>
+      <c r="L8" t="b">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8" t="b">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>0</v>
+      </c>
+      <c r="P8" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2">
+        <v>45868</v>
+      </c>
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+      <c r="E9" s="1">
+        <v>10000000</v>
+      </c>
+      <c r="F9">
+        <v>2.5000000000000001E-4</v>
+      </c>
+      <c r="G9">
+        <v>2048</v>
+      </c>
+      <c r="H9">
+        <v>4</v>
+      </c>
+      <c r="I9">
+        <v>0.1</v>
+      </c>
+      <c r="J9">
+        <v>0.01</v>
+      </c>
+      <c r="K9">
+        <v>0.95</v>
+      </c>
+      <c r="L9" t="b">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="N9" t="b">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>0</v>
+      </c>
+      <c r="P9" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q9">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: Add common evaluation interface for agents
Implemented set_eval_mode(), set_train_mode(), and get_greedy_action() methods in both DQN and PPO agents to create a unified interface for the evaluation script.

Removed early exploratory programs that have since been replaced.
</commit_message>
<xml_diff>
--- a/Eval_Run_Logs.xlsx
+++ b/Eval_Run_Logs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\DeepRL-MsPacman\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A01C34EB-9AB2-4A38-A3D1-832E0371793A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC6D8447-B71B-4B04-BCD5-5F5EE6B176A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{0D67D52D-1513-48BB-A273-B9082DA3F499}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{0D67D52D-1513-48BB-A273-B9082DA3F499}"/>
   </bookViews>
   <sheets>
     <sheet name="DQN_Runs" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="53">
   <si>
     <t>Run ID</t>
   </si>
@@ -190,6 +190,12 @@
   </si>
   <si>
     <t>PPO Baseline - 10M steps - High n_steps</t>
+  </si>
+  <si>
+    <t>DQN Baseline - 10M steps - Low Replay Buffer</t>
+  </si>
+  <si>
+    <t>PPO Baseline - 10M steps - High clip epsilon</t>
   </si>
 </sst>
 </file>
@@ -576,7 +582,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BDCA7AB-C83E-496B-A323-D25B7B27B0B8}">
-  <dimension ref="A1:V9"/>
+  <dimension ref="A1:V10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
@@ -1035,14 +1041,94 @@
         <v>0</v>
       </c>
     </row>
+    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2">
+        <v>45861</v>
+      </c>
+      <c r="C10" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="1">
+        <v>10000000</v>
+      </c>
+      <c r="F10">
+        <v>1E-4</v>
+      </c>
+      <c r="G10" s="1">
+        <v>100000</v>
+      </c>
+      <c r="H10" s="1">
+        <v>1000000</v>
+      </c>
+      <c r="I10" s="1">
+        <v>10000</v>
+      </c>
+      <c r="J10" t="b">
+        <v>0</v>
+      </c>
+      <c r="K10">
+        <v>0</v>
+      </c>
+      <c r="L10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10" t="b">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="F2:F10">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H10">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I10">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{606356CF-33ED-426F-8480-D5D1647FF48E}">
-  <dimension ref="A1:X9"/>
+  <dimension ref="A1:X10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
@@ -1557,7 +1643,93 @@
         <v>0</v>
       </c>
     </row>
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2">
+        <v>45869</v>
+      </c>
+      <c r="C10" t="s">
+        <v>52</v>
+      </c>
+      <c r="E10" s="1">
+        <v>10000000</v>
+      </c>
+      <c r="F10">
+        <v>2.5000000000000001E-4</v>
+      </c>
+      <c r="G10">
+        <v>128</v>
+      </c>
+      <c r="H10">
+        <v>4</v>
+      </c>
+      <c r="I10">
+        <v>0.3</v>
+      </c>
+      <c r="J10">
+        <v>0.01</v>
+      </c>
+      <c r="K10">
+        <v>0.95</v>
+      </c>
+      <c r="L10" t="b">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10" t="b">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>0</v>
+      </c>
+      <c r="P10" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="F2:F10">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G10">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H10">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added docstring to top of train.py
Ran and collected data from Evaluation_and_Analysis.ipynb
</commit_message>
<xml_diff>
--- a/Eval_Run_Logs.xlsx
+++ b/Eval_Run_Logs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\DeepRL-MsPacman\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC6D8447-B71B-4B04-BCD5-5F5EE6B176A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{475F1099-6632-4A31-940D-A75F280A47AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{0D67D52D-1513-48BB-A273-B9082DA3F499}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{0D67D52D-1513-48BB-A273-B9082DA3F499}"/>
   </bookViews>
   <sheets>
     <sheet name="DQN_Runs" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="58">
   <si>
     <t>Run ID</t>
   </si>
@@ -84,27 +84,6 @@
     <t>time_penalty_per_step</t>
   </si>
   <si>
-    <t>Mean Score (Eval)</t>
-  </si>
-  <si>
-    <t>Std Dev Score (Eval)</t>
-  </si>
-  <si>
-    <t>Median Score (Eval)</t>
-  </si>
-  <si>
-    <t>Max Score (Eval)</t>
-  </si>
-  <si>
-    <t>Level 1 Completion Rate (%)</t>
-  </si>
-  <si>
-    <t>Max Level Reached</t>
-  </si>
-  <si>
-    <t>Notes</t>
-  </si>
-  <si>
     <t>DQN Baseline - 10M steps, death penalty -250</t>
   </si>
   <si>
@@ -196,15 +175,52 @@
   </si>
   <si>
     <t>PPO Baseline - 10M steps - High clip epsilon</t>
+  </si>
+  <si>
+    <t>mean_score</t>
+  </si>
+  <si>
+    <t>std_score</t>
+  </si>
+  <si>
+    <t>min_score</t>
+  </si>
+  <si>
+    <t>Q1_score</t>
+  </si>
+  <si>
+    <t>Median_score</t>
+  </si>
+  <si>
+    <t>Q3_score</t>
+  </si>
+  <si>
+    <t>max_score</t>
+  </si>
+  <si>
+    <t>mean_steps</t>
+  </si>
+  <si>
+    <t>std_steps</t>
+  </si>
+  <si>
+    <t>level_1_completion_rate</t>
+  </si>
+  <si>
+    <t>mean_level_reached</t>
+  </si>
+  <si>
+    <t>max_level_reached</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="171" formatCode="0.0"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -243,10 +259,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -582,7 +600,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BDCA7AB-C83E-496B-A323-D25B7B27B0B8}">
-  <dimension ref="A1:V10"/>
+  <dimension ref="A1:AA10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
@@ -600,16 +618,18 @@
     <col min="13" max="13" width="22.7109375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="13.42578125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="9.140625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="9.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -656,28 +676,43 @@
         <v>14</v>
       </c>
       <c r="P1" t="s">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="Q1" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="R1" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
       <c r="S1" t="s">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="T1" t="s">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="U1" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="V1" t="s">
-        <v>21</v>
+        <v>52</v>
+      </c>
+      <c r="W1" t="s">
+        <v>53</v>
+      </c>
+      <c r="X1" t="s">
+        <v>54</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>55</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -685,10 +720,10 @@
         <v>45861</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="E2" s="1">
         <v>10000000</v>
@@ -723,8 +758,44 @@
       <c r="O2">
         <v>0</v>
       </c>
+      <c r="P2">
+        <v>2469.5</v>
+      </c>
+      <c r="Q2" s="3">
+        <v>546.14604736325305</v>
+      </c>
+      <c r="R2">
+        <v>1000</v>
+      </c>
+      <c r="S2">
+        <v>2160</v>
+      </c>
+      <c r="T2">
+        <v>2490</v>
+      </c>
+      <c r="U2">
+        <v>2792.5</v>
+      </c>
+      <c r="V2">
+        <v>4060</v>
+      </c>
+      <c r="W2">
+        <v>818.94</v>
+      </c>
+      <c r="X2" s="3">
+        <v>128.22500898534901</v>
+      </c>
+      <c r="Y2">
+        <v>0</v>
+      </c>
+      <c r="Z2">
+        <v>0</v>
+      </c>
+      <c r="AA2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -732,10 +803,10 @@
         <v>45861</v>
       </c>
       <c r="C3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="E3" s="1">
         <v>10000000</v>
@@ -770,8 +841,44 @@
       <c r="O3">
         <v>0</v>
       </c>
+      <c r="P3">
+        <v>3334.4</v>
+      </c>
+      <c r="Q3" s="3">
+        <v>904.977615661561</v>
+      </c>
+      <c r="R3">
+        <v>2290</v>
+      </c>
+      <c r="S3">
+        <v>2717.5</v>
+      </c>
+      <c r="T3">
+        <v>3025</v>
+      </c>
+      <c r="U3">
+        <v>3745</v>
+      </c>
+      <c r="V3">
+        <v>5810</v>
+      </c>
+      <c r="W3">
+        <v>900.88</v>
+      </c>
+      <c r="X3" s="3">
+        <v>131.220477584002</v>
+      </c>
+      <c r="Y3">
+        <v>0</v>
+      </c>
+      <c r="Z3">
+        <v>0</v>
+      </c>
+      <c r="AA3">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -779,10 +886,10 @@
         <v>45862</v>
       </c>
       <c r="C4" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="E4" s="1">
         <v>10000000</v>
@@ -817,8 +924,44 @@
       <c r="O4">
         <v>0</v>
       </c>
+      <c r="P4">
+        <v>3223.5</v>
+      </c>
+      <c r="Q4" s="3">
+        <v>804.45147256821599</v>
+      </c>
+      <c r="R4">
+        <v>1830</v>
+      </c>
+      <c r="S4">
+        <v>2780</v>
+      </c>
+      <c r="T4">
+        <v>3050</v>
+      </c>
+      <c r="U4">
+        <v>3345</v>
+      </c>
+      <c r="V4">
+        <v>6350</v>
+      </c>
+      <c r="W4">
+        <v>950.02</v>
+      </c>
+      <c r="X4" s="3">
+        <v>133.19037639272699</v>
+      </c>
+      <c r="Y4">
+        <v>0</v>
+      </c>
+      <c r="Z4">
+        <v>0</v>
+      </c>
+      <c r="AA4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -826,10 +969,10 @@
         <v>45865</v>
       </c>
       <c r="C5" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="E5" s="1">
         <v>10000000</v>
@@ -864,8 +1007,44 @@
       <c r="O5">
         <v>0</v>
       </c>
+      <c r="P5">
+        <v>2713.6</v>
+      </c>
+      <c r="Q5" s="3">
+        <v>575.54632807235896</v>
+      </c>
+      <c r="R5">
+        <v>1410</v>
+      </c>
+      <c r="S5">
+        <v>2410</v>
+      </c>
+      <c r="T5">
+        <v>2660</v>
+      </c>
+      <c r="U5">
+        <v>2955</v>
+      </c>
+      <c r="V5">
+        <v>5540</v>
+      </c>
+      <c r="W5">
+        <v>749.06</v>
+      </c>
+      <c r="X5" s="3">
+        <v>136.074980815873</v>
+      </c>
+      <c r="Y5">
+        <v>0</v>
+      </c>
+      <c r="Z5">
+        <v>0</v>
+      </c>
+      <c r="AA5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -873,7 +1052,7 @@
         <v>45866</v>
       </c>
       <c r="C6" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="E6" s="1">
         <v>10000000</v>
@@ -908,8 +1087,44 @@
       <c r="O6">
         <v>0</v>
       </c>
+      <c r="P6">
+        <v>3258.2</v>
+      </c>
+      <c r="Q6" s="3">
+        <v>833.37258089395903</v>
+      </c>
+      <c r="R6">
+        <v>2170</v>
+      </c>
+      <c r="S6">
+        <v>2487.5</v>
+      </c>
+      <c r="T6">
+        <v>3130</v>
+      </c>
+      <c r="U6">
+        <v>3975</v>
+      </c>
+      <c r="V6">
+        <v>5360</v>
+      </c>
+      <c r="W6">
+        <v>841.72</v>
+      </c>
+      <c r="X6" s="3">
+        <v>157.91380336414301</v>
+      </c>
+      <c r="Y6">
+        <v>0</v>
+      </c>
+      <c r="Z6">
+        <v>0</v>
+      </c>
+      <c r="AA6">
+        <v>0</v>
+      </c>
     </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -917,7 +1132,7 @@
         <v>45861</v>
       </c>
       <c r="C7" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="E7" s="1">
         <v>10000000</v>
@@ -952,8 +1167,44 @@
       <c r="O7">
         <v>0</v>
       </c>
+      <c r="P7">
+        <v>3477.2</v>
+      </c>
+      <c r="Q7" s="3">
+        <v>900.75622550042795</v>
+      </c>
+      <c r="R7">
+        <v>2300</v>
+      </c>
+      <c r="S7">
+        <v>2835</v>
+      </c>
+      <c r="T7">
+        <v>3090</v>
+      </c>
+      <c r="U7">
+        <v>4110</v>
+      </c>
+      <c r="V7">
+        <v>5530</v>
+      </c>
+      <c r="W7">
+        <v>913.56</v>
+      </c>
+      <c r="X7" s="3">
+        <v>135.12346168963299</v>
+      </c>
+      <c r="Y7">
+        <v>0</v>
+      </c>
+      <c r="Z7">
+        <v>0</v>
+      </c>
+      <c r="AA7">
+        <v>0</v>
+      </c>
     </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -961,7 +1212,7 @@
         <v>45861</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="E8" s="1">
         <v>10000000</v>
@@ -996,8 +1247,44 @@
       <c r="O8">
         <v>0</v>
       </c>
+      <c r="P8">
+        <v>2451.4</v>
+      </c>
+      <c r="Q8" s="3">
+        <v>966.69176560937399</v>
+      </c>
+      <c r="R8">
+        <v>420</v>
+      </c>
+      <c r="S8">
+        <v>1697.5</v>
+      </c>
+      <c r="T8">
+        <v>2515</v>
+      </c>
+      <c r="U8">
+        <v>2865</v>
+      </c>
+      <c r="V8">
+        <v>5540</v>
+      </c>
+      <c r="W8">
+        <v>859.82</v>
+      </c>
+      <c r="X8" s="3">
+        <v>119.96501005027901</v>
+      </c>
+      <c r="Y8">
+        <v>0</v>
+      </c>
+      <c r="Z8">
+        <v>0</v>
+      </c>
+      <c r="AA8">
+        <v>0</v>
+      </c>
     </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1005,7 +1292,7 @@
         <v>45861</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="E9" s="1">
         <v>10000000</v>
@@ -1040,8 +1327,44 @@
       <c r="O9">
         <v>0</v>
       </c>
+      <c r="P9">
+        <v>2132</v>
+      </c>
+      <c r="Q9" s="3">
+        <v>760.62441122376197</v>
+      </c>
+      <c r="R9">
+        <v>960</v>
+      </c>
+      <c r="S9">
+        <v>1555</v>
+      </c>
+      <c r="T9">
+        <v>1960</v>
+      </c>
+      <c r="U9">
+        <v>2557.5</v>
+      </c>
+      <c r="V9">
+        <v>4540</v>
+      </c>
+      <c r="W9">
+        <v>902</v>
+      </c>
+      <c r="X9" s="3">
+        <v>123.834200005124</v>
+      </c>
+      <c r="Y9">
+        <v>0</v>
+      </c>
+      <c r="Z9">
+        <v>0</v>
+      </c>
+      <c r="AA9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1049,7 +1372,7 @@
         <v>45861</v>
       </c>
       <c r="C10" t="s">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="E10" s="1">
         <v>10000000</v>
@@ -1087,6 +1410,114 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F10">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H10">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I10">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P2:P10">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q2:Q10">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R2:R10">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S2:S10">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T2:T10">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U2:U10">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V2:V10">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -1098,7 +1529,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H10">
+  <conditionalFormatting sqref="W2:W10">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -1110,7 +1541,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I10">
+  <conditionalFormatting sqref="X2:X10">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1128,7 +1559,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{606356CF-33ED-426F-8480-D5D1647FF48E}">
-  <dimension ref="A1:X10"/>
+  <dimension ref="A1:AC10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
@@ -1148,16 +1579,17 @@
     <col min="15" max="15" width="22.7109375" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="20.7109375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="25.5703125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="17.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="9.140625" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="22.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1177,19 +1609,19 @@
         <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="H1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="I1" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="J1" t="s">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="K1" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="L1" t="s">
         <v>9</v>
@@ -1210,28 +1642,43 @@
         <v>14</v>
       </c>
       <c r="R1" t="s">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="S1" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="T1" t="s">
-        <v>17</v>
+        <v>48</v>
       </c>
       <c r="U1" t="s">
-        <v>18</v>
+        <v>49</v>
       </c>
       <c r="V1" t="s">
-        <v>19</v>
+        <v>50</v>
       </c>
       <c r="W1" t="s">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="X1" t="s">
-        <v>21</v>
+        <v>52</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>53</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>54</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>55</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>56</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>57</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1239,10 +1686,10 @@
         <v>45861</v>
       </c>
       <c r="C2" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="E2" s="1">
         <v>10000000</v>
@@ -1283,8 +1730,44 @@
       <c r="Q2">
         <v>0</v>
       </c>
+      <c r="R2" s="4">
+        <v>210</v>
+      </c>
+      <c r="S2" s="3">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>210</v>
+      </c>
+      <c r="U2">
+        <v>210</v>
+      </c>
+      <c r="V2">
+        <v>210</v>
+      </c>
+      <c r="W2">
+        <v>210</v>
+      </c>
+      <c r="X2">
+        <v>210</v>
+      </c>
+      <c r="Y2">
+        <v>735</v>
+      </c>
+      <c r="Z2">
+        <v>0</v>
+      </c>
+      <c r="AA2">
+        <v>0</v>
+      </c>
+      <c r="AB2">
+        <v>0</v>
+      </c>
+      <c r="AC2">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1292,10 +1775,10 @@
         <v>45862</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="E3" s="1">
         <v>10000000</v>
@@ -1336,8 +1819,44 @@
       <c r="Q3">
         <v>-1</v>
       </c>
+      <c r="R3" s="4">
+        <v>757.9</v>
+      </c>
+      <c r="S3" s="3">
+        <v>47.445769148586997</v>
+      </c>
+      <c r="T3">
+        <v>690</v>
+      </c>
+      <c r="U3">
+        <v>750</v>
+      </c>
+      <c r="V3">
+        <v>750</v>
+      </c>
+      <c r="W3">
+        <v>780</v>
+      </c>
+      <c r="X3">
+        <v>1120</v>
+      </c>
+      <c r="Y3">
+        <v>616.32000000000005</v>
+      </c>
+      <c r="Z3">
+        <v>46.862981018059301</v>
+      </c>
+      <c r="AA3">
+        <v>0</v>
+      </c>
+      <c r="AB3">
+        <v>0</v>
+      </c>
+      <c r="AC3">
+        <v>0</v>
+      </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1345,10 +1864,10 @@
         <v>45862</v>
       </c>
       <c r="C4" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="E4" s="1">
         <v>10000000</v>
@@ -1389,8 +1908,44 @@
       <c r="Q4">
         <v>0</v>
       </c>
+      <c r="R4" s="4">
+        <v>70</v>
+      </c>
+      <c r="S4" s="3">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>70</v>
+      </c>
+      <c r="U4">
+        <v>70</v>
+      </c>
+      <c r="V4">
+        <v>70</v>
+      </c>
+      <c r="W4">
+        <v>70</v>
+      </c>
+      <c r="X4">
+        <v>70</v>
+      </c>
+      <c r="Y4">
+        <v>529</v>
+      </c>
+      <c r="Z4">
+        <v>0</v>
+      </c>
+      <c r="AA4">
+        <v>0</v>
+      </c>
+      <c r="AB4">
+        <v>0</v>
+      </c>
+      <c r="AC4">
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1398,10 +1953,10 @@
         <v>45865</v>
       </c>
       <c r="C5" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="D5" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="E5" s="1">
         <v>10000000</v>
@@ -1442,8 +1997,44 @@
       <c r="Q5">
         <v>0</v>
       </c>
+      <c r="R5" s="4">
+        <v>168.8</v>
+      </c>
+      <c r="S5" s="3">
+        <v>11.8304520606609</v>
+      </c>
+      <c r="T5">
+        <v>120</v>
+      </c>
+      <c r="U5">
+        <v>170</v>
+      </c>
+      <c r="V5">
+        <v>170</v>
+      </c>
+      <c r="W5">
+        <v>170</v>
+      </c>
+      <c r="X5">
+        <v>240</v>
+      </c>
+      <c r="Y5">
+        <v>557.04</v>
+      </c>
+      <c r="Z5">
+        <v>9.6775487337935608</v>
+      </c>
+      <c r="AA5">
+        <v>0</v>
+      </c>
+      <c r="AB5">
+        <v>0</v>
+      </c>
+      <c r="AC5">
+        <v>0</v>
+      </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1451,7 +2042,7 @@
         <v>45866</v>
       </c>
       <c r="C6" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E6" s="1">
         <v>10000000</v>
@@ -1492,8 +2083,44 @@
       <c r="Q6">
         <v>0</v>
       </c>
+      <c r="R6" s="4">
+        <v>820</v>
+      </c>
+      <c r="S6" s="3">
+        <v>0</v>
+      </c>
+      <c r="T6">
+        <v>820</v>
+      </c>
+      <c r="U6">
+        <v>820</v>
+      </c>
+      <c r="V6">
+        <v>820</v>
+      </c>
+      <c r="W6">
+        <v>820</v>
+      </c>
+      <c r="X6">
+        <v>820</v>
+      </c>
+      <c r="Y6">
+        <v>729</v>
+      </c>
+      <c r="Z6">
+        <v>0</v>
+      </c>
+      <c r="AA6">
+        <v>0</v>
+      </c>
+      <c r="AB6">
+        <v>0</v>
+      </c>
+      <c r="AC6">
+        <v>0</v>
+      </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1501,7 +2128,7 @@
         <v>45867</v>
       </c>
       <c r="C7" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="E7" s="1">
         <v>10000000</v>
@@ -1542,8 +2169,44 @@
       <c r="Q7">
         <v>0</v>
       </c>
+      <c r="R7" s="4">
+        <v>70</v>
+      </c>
+      <c r="S7" s="3">
+        <v>0</v>
+      </c>
+      <c r="T7">
+        <v>70</v>
+      </c>
+      <c r="U7">
+        <v>70</v>
+      </c>
+      <c r="V7">
+        <v>70</v>
+      </c>
+      <c r="W7">
+        <v>70</v>
+      </c>
+      <c r="X7">
+        <v>70</v>
+      </c>
+      <c r="Y7">
+        <v>529</v>
+      </c>
+      <c r="Z7">
+        <v>0</v>
+      </c>
+      <c r="AA7">
+        <v>0</v>
+      </c>
+      <c r="AB7">
+        <v>0</v>
+      </c>
+      <c r="AC7">
+        <v>0</v>
+      </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1551,7 +2214,7 @@
         <v>45868</v>
       </c>
       <c r="C8" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="E8" s="1">
         <v>10000000</v>
@@ -1592,8 +2255,44 @@
       <c r="Q8">
         <v>0</v>
       </c>
+      <c r="R8" s="4">
+        <v>1084.4000000000001</v>
+      </c>
+      <c r="S8" s="3">
+        <v>184.14048216434401</v>
+      </c>
+      <c r="T8">
+        <v>770</v>
+      </c>
+      <c r="U8">
+        <v>1170</v>
+      </c>
+      <c r="V8">
+        <v>1170</v>
+      </c>
+      <c r="W8">
+        <v>1170</v>
+      </c>
+      <c r="X8">
+        <v>1810</v>
+      </c>
+      <c r="Y8">
+        <v>623.1</v>
+      </c>
+      <c r="Z8">
+        <v>1</v>
+      </c>
+      <c r="AA8">
+        <v>0</v>
+      </c>
+      <c r="AB8">
+        <v>0</v>
+      </c>
+      <c r="AC8">
+        <v>0</v>
+      </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1601,7 +2300,7 @@
         <v>45868</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="E9" s="1">
         <v>10000000</v>
@@ -1642,8 +2341,44 @@
       <c r="Q9">
         <v>0</v>
       </c>
+      <c r="R9" s="4">
+        <v>232.2</v>
+      </c>
+      <c r="S9" s="3">
+        <v>7.8598840817010602</v>
+      </c>
+      <c r="T9">
+        <v>200</v>
+      </c>
+      <c r="U9">
+        <v>230</v>
+      </c>
+      <c r="V9">
+        <v>230</v>
+      </c>
+      <c r="W9">
+        <v>240</v>
+      </c>
+      <c r="X9">
+        <v>240</v>
+      </c>
+      <c r="Y9">
+        <v>493.2</v>
+      </c>
+      <c r="Z9">
+        <v>2.1367397047035301</v>
+      </c>
+      <c r="AA9">
+        <v>0</v>
+      </c>
+      <c r="AB9">
+        <v>0</v>
+      </c>
+      <c r="AC9">
+        <v>0</v>
+      </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
@@ -1651,7 +2386,7 @@
         <v>45869</v>
       </c>
       <c r="C10" t="s">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="E10" s="1">
         <v>10000000</v>
@@ -1695,6 +2430,102 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F10">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G10">
+    <cfRule type="colorScale" priority="15">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H10">
+    <cfRule type="colorScale" priority="17">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R2:R10">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S2:S10">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T2:T10">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U2:U10">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V2:V10">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W2:W10">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -1706,8 +2537,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G10">
-    <cfRule type="colorScale" priority="6">
+  <conditionalFormatting sqref="X2:X10">
+    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1718,8 +2549,20 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H10">
-    <cfRule type="colorScale" priority="8">
+  <conditionalFormatting sqref="Y2:Y10">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z2:Z10">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>

<commit_message>
style: Document and polish core trainin/evaluation scripts
This commit focuses on improving code quality, documentation, and robustness across the main project scripts.
</commit_message>
<xml_diff>
--- a/Eval_Run_Logs.xlsx
+++ b/Eval_Run_Logs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\DeepRL-MsPacman\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{475F1099-6632-4A31-940D-A75F280A47AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46831F99-F396-4B95-956C-1719F2D4757A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{0D67D52D-1513-48BB-A273-B9082DA3F499}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="72">
   <si>
     <t>Run ID</t>
   </si>
@@ -211,6 +211,48 @@
   </si>
   <si>
     <t>max_level_reached</t>
+  </si>
+  <si>
+    <t>PPO Baseline - 10M steps - High Entropy Coeff</t>
+  </si>
+  <si>
+    <t>DQN Baseline - 10M steps - High Replay Buffer</t>
+  </si>
+  <si>
+    <t>Notes:</t>
+  </si>
+  <si>
+    <t>250k buffer costs 10GB of RAM, 500k costs 20 GB</t>
+  </si>
+  <si>
+    <t>We might be able to do 750k buffer if performance boost warents, but need to check on RAM use of Reward shaping features</t>
+  </si>
+  <si>
+    <t>Optimal</t>
+  </si>
+  <si>
+    <t>Med n_step</t>
+  </si>
+  <si>
+    <t>med_LR</t>
+  </si>
+  <si>
+    <t>Low_Epochs</t>
+  </si>
+  <si>
+    <t>High clip</t>
+  </si>
+  <si>
+    <t>High Entropy</t>
+  </si>
+  <si>
+    <t>Baseline Epsilon Decay</t>
+  </si>
+  <si>
+    <t>Baseline Update Freq</t>
+  </si>
+  <si>
+    <t>High LR</t>
   </si>
 </sst>
 </file>
@@ -220,7 +262,7 @@
   <numFmts count="3">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
-    <numFmt numFmtId="171" formatCode="0.0"/>
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -259,12 +301,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -600,7 +645,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BDCA7AB-C83E-496B-A323-D25B7B27B0B8}">
-  <dimension ref="A1:AA10"/>
+  <dimension ref="A1:AA23"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
@@ -1289,7 +1334,7 @@
         <v>8</v>
       </c>
       <c r="B9" s="2">
-        <v>45861</v>
+        <v>45869</v>
       </c>
       <c r="C9" t="s">
         <v>42</v>
@@ -1369,7 +1414,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="2">
-        <v>45861</v>
+        <v>45870</v>
       </c>
       <c r="C10" t="s">
         <v>44</v>
@@ -1408,8 +1453,97 @@
         <v>0</v>
       </c>
     </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2">
+        <v>45871</v>
+      </c>
+      <c r="C11" t="s">
+        <v>59</v>
+      </c>
+      <c r="E11" s="1">
+        <v>10000000</v>
+      </c>
+      <c r="F11">
+        <v>1E-4</v>
+      </c>
+      <c r="G11" s="1">
+        <v>500000</v>
+      </c>
+      <c r="H11" s="1">
+        <v>1000000</v>
+      </c>
+      <c r="I11" s="1">
+        <v>10000</v>
+      </c>
+      <c r="J11" t="b">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11" t="b">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="N11" t="b">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>60</v>
+      </c>
+      <c r="C17" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18" spans="2:3" ht="45" x14ac:dyDescent="0.25">
+      <c r="C18" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="20" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C20" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="21" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="22" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="23" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="C23" t="s">
+        <v>71</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:F10">
+  <conditionalFormatting sqref="F2:F11">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H11">
     <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="min"/>
@@ -1421,7 +1555,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H10">
+  <conditionalFormatting sqref="I2:I11">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -1433,7 +1567,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I10">
+  <conditionalFormatting sqref="P2:P11">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
@@ -1445,7 +1579,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P10">
+  <conditionalFormatting sqref="Q2:Q11">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -1457,7 +1591,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Q2:Q10">
+  <conditionalFormatting sqref="R2:R11">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -1469,7 +1603,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R2:R10">
+  <conditionalFormatting sqref="S2:S11">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -1481,7 +1615,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S10">
+  <conditionalFormatting sqref="T2:T11">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -1493,7 +1627,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T2:T10">
+  <conditionalFormatting sqref="U2:U11">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -1505,7 +1639,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U2:U10">
+  <conditionalFormatting sqref="V2:V11">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -1517,7 +1651,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V2:V10">
+  <conditionalFormatting sqref="W2:W11">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -1529,7 +1663,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W2:W10">
+  <conditionalFormatting sqref="X2:X11">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -1541,7 +1675,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X2:X10">
+  <conditionalFormatting sqref="G2:G11">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1559,7 +1693,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{606356CF-33ED-426F-8480-D5D1647FF48E}">
-  <dimension ref="A1:AC10"/>
+  <dimension ref="A1:AC25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
@@ -2428,20 +2562,88 @@
         <v>0</v>
       </c>
     </row>
+    <row r="11" spans="1:29" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2">
+        <v>45869</v>
+      </c>
+      <c r="C11" t="s">
+        <v>58</v>
+      </c>
+      <c r="E11" s="1">
+        <v>10000000</v>
+      </c>
+      <c r="F11">
+        <v>2.5000000000000001E-4</v>
+      </c>
+      <c r="G11">
+        <v>128</v>
+      </c>
+      <c r="H11">
+        <v>4</v>
+      </c>
+      <c r="I11">
+        <v>0.1</v>
+      </c>
+      <c r="J11">
+        <v>0.05</v>
+      </c>
+      <c r="K11">
+        <v>0.95</v>
+      </c>
+      <c r="L11" t="b">
+        <v>0</v>
+      </c>
+      <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="N11" t="b">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C20" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="21" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C21" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="22" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C22" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="23" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C23" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="24" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C24" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="25" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C25" t="s">
+        <v>68</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:F10">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G10">
+  <conditionalFormatting sqref="F2:F11">
     <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
@@ -2453,7 +2655,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H10">
+  <conditionalFormatting sqref="G2:G11">
     <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="min"/>
@@ -2465,7 +2667,43 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="R2:R10">
+  <conditionalFormatting sqref="H2:H11">
+    <cfRule type="colorScale" priority="19">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R2:R11">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S2:S11">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="T2:T11">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -2477,7 +2715,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S10">
+  <conditionalFormatting sqref="U2:U11">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -2489,7 +2727,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T2:T10">
+  <conditionalFormatting sqref="V2:V11">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -2501,7 +2739,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U2:U10">
+  <conditionalFormatting sqref="W2:W11">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -2513,7 +2751,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V2:V10">
+  <conditionalFormatting sqref="X2:X11">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -2525,7 +2763,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W2:W10">
+  <conditionalFormatting sqref="Y2:Y11">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -2537,7 +2775,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X2:X10">
+  <conditionalFormatting sqref="Z2:Z11">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -2549,7 +2787,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Y2:Y10">
+  <conditionalFormatting sqref="I2:I11">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -2561,7 +2799,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Z2:Z10">
+  <conditionalFormatting sqref="J2:J11">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
style: Document and polish all core project modles
This commit completes a comprehensive code quality review.
</commit_message>
<xml_diff>
--- a/Eval_Run_Logs.xlsx
+++ b/Eval_Run_Logs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\DeepRL-MsPacman\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46831F99-F396-4B95-956C-1719F2D4757A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{604CCDE6-276A-44F5-8776-B7317CE82452}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="25440" windowHeight="15270" activeTab="1" xr2:uid="{0D67D52D-1513-48BB-A273-B9082DA3F499}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{0D67D52D-1513-48BB-A273-B9082DA3F499}"/>
   </bookViews>
   <sheets>
     <sheet name="DQN_Runs" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="73">
   <si>
     <t>Run ID</t>
   </si>
@@ -253,6 +253,9 @@
   </si>
   <si>
     <t>High LR</t>
+  </si>
+  <si>
+    <t>DQN Baseline - 10M steps - Very High LR</t>
   </si>
 </sst>
 </file>
@@ -804,31 +807,31 @@
         <v>0</v>
       </c>
       <c r="P2">
-        <v>2469.5</v>
+        <v>2580.5</v>
       </c>
       <c r="Q2" s="3">
-        <v>546.14604736325305</v>
+        <v>656.08997714965301</v>
       </c>
       <c r="R2">
-        <v>1000</v>
+        <v>1360</v>
       </c>
       <c r="S2">
-        <v>2160</v>
+        <v>2227.5</v>
       </c>
       <c r="T2">
-        <v>2490</v>
+        <v>2530</v>
       </c>
       <c r="U2">
-        <v>2792.5</v>
+        <v>2920</v>
       </c>
       <c r="V2">
-        <v>4060</v>
+        <v>6220</v>
       </c>
       <c r="W2">
-        <v>818.94</v>
+        <v>830.82399999999996</v>
       </c>
       <c r="X2" s="3">
-        <v>128.22500898534901</v>
+        <v>135.612087590307</v>
       </c>
       <c r="Y2">
         <v>0</v>
@@ -887,31 +890,31 @@
         <v>0</v>
       </c>
       <c r="P3">
-        <v>3334.4</v>
+        <v>3222.2</v>
       </c>
       <c r="Q3" s="3">
-        <v>904.977615661561</v>
+        <v>845.22326324436801</v>
       </c>
       <c r="R3">
-        <v>2290</v>
+        <v>2160</v>
       </c>
       <c r="S3">
-        <v>2717.5</v>
+        <v>2670</v>
       </c>
       <c r="T3">
-        <v>3025</v>
+        <v>2985</v>
       </c>
       <c r="U3">
-        <v>3745</v>
+        <v>3380</v>
       </c>
       <c r="V3">
-        <v>5810</v>
+        <v>8840</v>
       </c>
       <c r="W3">
-        <v>900.88</v>
+        <v>902.71600000000001</v>
       </c>
       <c r="X3" s="3">
-        <v>131.220477584002</v>
+        <v>126.13689538257</v>
       </c>
       <c r="Y3">
         <v>0</v>
@@ -970,31 +973,31 @@
         <v>0</v>
       </c>
       <c r="P4">
-        <v>3223.5</v>
+        <v>3069.3</v>
       </c>
       <c r="Q4" s="3">
-        <v>804.45147256821599</v>
+        <v>713.73310129190395</v>
       </c>
       <c r="R4">
-        <v>1830</v>
+        <v>1520</v>
       </c>
       <c r="S4">
-        <v>2780</v>
+        <v>2660</v>
       </c>
       <c r="T4">
-        <v>3050</v>
+        <v>2990</v>
       </c>
       <c r="U4">
-        <v>3345</v>
+        <v>3330</v>
       </c>
       <c r="V4">
-        <v>6350</v>
+        <v>5660</v>
       </c>
       <c r="W4">
-        <v>950.02</v>
+        <v>941.57600000000002</v>
       </c>
       <c r="X4" s="3">
-        <v>133.19037639272699</v>
+        <v>133.11126715227999</v>
       </c>
       <c r="Y4">
         <v>0</v>
@@ -1053,31 +1056,31 @@
         <v>0</v>
       </c>
       <c r="P5">
-        <v>2713.6</v>
+        <v>2735.14</v>
       </c>
       <c r="Q5" s="3">
-        <v>575.54632807235896</v>
+        <v>640.27782390425398</v>
       </c>
       <c r="R5">
-        <v>1410</v>
+        <v>1360</v>
       </c>
       <c r="S5">
-        <v>2410</v>
+        <v>2390</v>
       </c>
       <c r="T5">
-        <v>2660</v>
+        <v>2670</v>
       </c>
       <c r="U5">
-        <v>2955</v>
+        <v>2970</v>
       </c>
       <c r="V5">
-        <v>5540</v>
+        <v>6300</v>
       </c>
       <c r="W5">
-        <v>749.06</v>
+        <v>745.16399999999999</v>
       </c>
       <c r="X5" s="3">
-        <v>136.074980815873</v>
+        <v>125.934602680536</v>
       </c>
       <c r="Y5">
         <v>0</v>
@@ -1133,31 +1136,31 @@
         <v>0</v>
       </c>
       <c r="P6">
-        <v>3258.2</v>
+        <v>3350.14</v>
       </c>
       <c r="Q6" s="3">
-        <v>833.37258089395903</v>
+        <v>861.05296283656003</v>
       </c>
       <c r="R6">
-        <v>2170</v>
+        <v>2090</v>
       </c>
       <c r="S6">
-        <v>2487.5</v>
+        <v>2557.5</v>
       </c>
       <c r="T6">
-        <v>3130</v>
+        <v>3140</v>
       </c>
       <c r="U6">
-        <v>3975</v>
+        <v>4110</v>
       </c>
       <c r="V6">
-        <v>5360</v>
+        <v>6170</v>
       </c>
       <c r="W6">
-        <v>841.72</v>
+        <v>806.90800000000002</v>
       </c>
       <c r="X6" s="3">
-        <v>157.91380336414301</v>
+        <v>141.791343551757</v>
       </c>
       <c r="Y6">
         <v>0</v>
@@ -1213,31 +1216,31 @@
         <v>0</v>
       </c>
       <c r="P7">
-        <v>3477.2</v>
+        <v>3277.74</v>
       </c>
       <c r="Q7" s="3">
-        <v>900.75622550042795</v>
+        <v>867.61085146461699</v>
       </c>
       <c r="R7">
-        <v>2300</v>
+        <v>1760</v>
       </c>
       <c r="S7">
-        <v>2835</v>
+        <v>2610</v>
       </c>
       <c r="T7">
-        <v>3090</v>
+        <v>2990</v>
       </c>
       <c r="U7">
-        <v>4110</v>
+        <v>4070</v>
       </c>
       <c r="V7">
-        <v>5530</v>
+        <v>6760</v>
       </c>
       <c r="W7">
-        <v>913.56</v>
+        <v>912.06399999999996</v>
       </c>
       <c r="X7" s="3">
-        <v>135.12346168963299</v>
+        <v>121.67595481425199</v>
       </c>
       <c r="Y7">
         <v>0</v>
@@ -1293,31 +1296,31 @@
         <v>0</v>
       </c>
       <c r="P8">
-        <v>2451.4</v>
+        <v>2345.98</v>
       </c>
       <c r="Q8" s="3">
-        <v>966.69176560937399</v>
+        <v>787.898475449236</v>
       </c>
       <c r="R8">
-        <v>420</v>
+        <v>330</v>
       </c>
       <c r="S8">
-        <v>1697.5</v>
+        <v>1760</v>
       </c>
       <c r="T8">
-        <v>2515</v>
+        <v>2450</v>
       </c>
       <c r="U8">
-        <v>2865</v>
+        <v>2760</v>
       </c>
       <c r="V8">
-        <v>5540</v>
+        <v>5390</v>
       </c>
       <c r="W8">
-        <v>859.82</v>
+        <v>876.596</v>
       </c>
       <c r="X8" s="3">
-        <v>119.96501005027901</v>
+        <v>143.47668766669901</v>
       </c>
       <c r="Y8">
         <v>0</v>
@@ -1373,31 +1376,31 @@
         <v>0</v>
       </c>
       <c r="P9">
-        <v>2132</v>
+        <v>2088.36</v>
       </c>
       <c r="Q9" s="3">
-        <v>760.62441122376197</v>
+        <v>805.47805693290002</v>
       </c>
       <c r="R9">
-        <v>960</v>
+        <v>830</v>
       </c>
       <c r="S9">
-        <v>1555</v>
+        <v>1497.5</v>
       </c>
       <c r="T9">
-        <v>1960</v>
+        <v>1880</v>
       </c>
       <c r="U9">
-        <v>2557.5</v>
+        <v>2475</v>
       </c>
       <c r="V9">
-        <v>4540</v>
+        <v>5240</v>
       </c>
       <c r="W9">
-        <v>902</v>
+        <v>921.77200000000005</v>
       </c>
       <c r="X9" s="3">
-        <v>123.834200005124</v>
+        <v>122.177062024628</v>
       </c>
       <c r="Y9">
         <v>0</v>
@@ -1452,6 +1455,33 @@
       <c r="O10">
         <v>0</v>
       </c>
+      <c r="P10">
+        <v>2721.64</v>
+      </c>
+      <c r="Q10">
+        <v>718.89507625335796</v>
+      </c>
+      <c r="R10">
+        <v>1180</v>
+      </c>
+      <c r="S10">
+        <v>2300</v>
+      </c>
+      <c r="T10">
+        <v>2640</v>
+      </c>
+      <c r="U10">
+        <v>3040</v>
+      </c>
+      <c r="V10">
+        <v>6740</v>
+      </c>
+      <c r="W10">
+        <v>818.404</v>
+      </c>
+      <c r="X10">
+        <v>136.22434043096499</v>
+      </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11">
@@ -1496,6 +1526,77 @@
       <c r="O11">
         <v>0</v>
       </c>
+      <c r="P11">
+        <v>3231.52</v>
+      </c>
+      <c r="Q11">
+        <v>682.30254515592401</v>
+      </c>
+      <c r="R11">
+        <v>1870</v>
+      </c>
+      <c r="S11">
+        <v>2730</v>
+      </c>
+      <c r="T11">
+        <v>3080</v>
+      </c>
+      <c r="U11">
+        <v>3622.5</v>
+      </c>
+      <c r="V11">
+        <v>7360</v>
+      </c>
+      <c r="W11">
+        <v>891.82399999999996</v>
+      </c>
+      <c r="X11">
+        <v>125.895688857664</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2">
+        <v>45872</v>
+      </c>
+      <c r="C12" t="s">
+        <v>72</v>
+      </c>
+      <c r="E12" s="1">
+        <v>10000000</v>
+      </c>
+      <c r="F12">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="G12" s="1">
+        <v>250000</v>
+      </c>
+      <c r="H12" s="1">
+        <v>1000000</v>
+      </c>
+      <c r="I12" s="1">
+        <v>10000</v>
+      </c>
+      <c r="J12" t="b">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12" t="b">
+        <v>0</v>
+      </c>
+      <c r="M12">
+        <v>0</v>
+      </c>
+      <c r="N12" t="b">
+        <v>0</v>
+      </c>
+      <c r="O12">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
@@ -1531,7 +1632,7 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:F11">
+  <conditionalFormatting sqref="F2:F12">
     <cfRule type="colorScale" priority="13">
       <colorScale>
         <cfvo type="min"/>
@@ -1543,7 +1644,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H11">
+  <conditionalFormatting sqref="H2:H12">
     <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="min"/>
@@ -1555,7 +1656,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I11">
+  <conditionalFormatting sqref="I2:I12">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -1675,7 +1776,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G11">
+  <conditionalFormatting sqref="G2:G12">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1954,16 +2055,16 @@
         <v>-1</v>
       </c>
       <c r="R3" s="4">
-        <v>757.9</v>
+        <v>752.16</v>
       </c>
       <c r="S3" s="3">
-        <v>47.445769148586997</v>
+        <v>50.039407316325502</v>
       </c>
       <c r="T3">
         <v>690</v>
       </c>
       <c r="U3">
-        <v>750</v>
+        <v>710</v>
       </c>
       <c r="V3">
         <v>750</v>
@@ -1972,13 +2073,13 @@
         <v>780</v>
       </c>
       <c r="X3">
-        <v>1120</v>
+        <v>1400</v>
       </c>
       <c r="Y3">
-        <v>616.32000000000005</v>
+        <v>618.54399999999998</v>
       </c>
       <c r="Z3">
-        <v>46.862981018059301</v>
+        <v>58.606257779368597</v>
       </c>
       <c r="AA3">
         <v>0</v>
@@ -2132,10 +2233,10 @@
         <v>0</v>
       </c>
       <c r="R5" s="4">
-        <v>168.8</v>
+        <v>168.34</v>
       </c>
       <c r="S5" s="3">
-        <v>11.8304520606609</v>
+        <v>9.3819209590447699</v>
       </c>
       <c r="T5">
         <v>120</v>
@@ -2153,10 +2254,10 @@
         <v>240</v>
       </c>
       <c r="Y5">
-        <v>557.04</v>
+        <v>556.65599999999995</v>
       </c>
       <c r="Z5">
-        <v>9.6775487337935608</v>
+        <v>10.6438831493489</v>
       </c>
       <c r="AA5">
         <v>0</v>
@@ -2390,16 +2491,16 @@
         <v>0</v>
       </c>
       <c r="R8" s="4">
-        <v>1084.4000000000001</v>
+        <v>1071.44</v>
       </c>
       <c r="S8" s="3">
-        <v>184.14048216434401</v>
+        <v>183.76906305761599</v>
       </c>
       <c r="T8">
         <v>770</v>
       </c>
       <c r="U8">
-        <v>1170</v>
+        <v>770</v>
       </c>
       <c r="V8">
         <v>1170</v>
@@ -2411,10 +2512,10 @@
         <v>1810</v>
       </c>
       <c r="Y8">
-        <v>623.1</v>
+        <v>623.05999999999995</v>
       </c>
       <c r="Z8">
-        <v>1</v>
+        <v>0.77304281277349796</v>
       </c>
       <c r="AA8">
         <v>0</v>
@@ -2476,10 +2577,10 @@
         <v>0</v>
       </c>
       <c r="R9" s="4">
-        <v>232.2</v>
+        <v>232.94</v>
       </c>
       <c r="S9" s="3">
-        <v>7.8598840817010602</v>
+        <v>7.8791218496888602</v>
       </c>
       <c r="T9">
         <v>200</v>
@@ -2497,10 +2598,10 @@
         <v>240</v>
       </c>
       <c r="Y9">
-        <v>493.2</v>
+        <v>493.20800000000003</v>
       </c>
       <c r="Z9">
-        <v>2.1367397047035301</v>
+        <v>1.7874916090726101</v>
       </c>
       <c r="AA9">
         <v>0</v>
@@ -2561,6 +2662,42 @@
       <c r="Q10">
         <v>0</v>
       </c>
+      <c r="R10">
+        <v>1135.54</v>
+      </c>
+      <c r="S10">
+        <v>211.281774833404</v>
+      </c>
+      <c r="T10">
+        <v>600</v>
+      </c>
+      <c r="U10">
+        <v>940</v>
+      </c>
+      <c r="V10">
+        <v>1250</v>
+      </c>
+      <c r="W10">
+        <v>1320</v>
+      </c>
+      <c r="X10">
+        <v>1600</v>
+      </c>
+      <c r="Y10">
+        <v>720.36</v>
+      </c>
+      <c r="Z10">
+        <v>169.13901505219201</v>
+      </c>
+      <c r="AA10">
+        <v>0</v>
+      </c>
+      <c r="AB10">
+        <v>0</v>
+      </c>
+      <c r="AC10">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.25">
       <c r="A11">
@@ -2611,39 +2748,138 @@
       <c r="Q11">
         <v>0</v>
       </c>
-    </row>
-    <row r="20" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="R11">
+        <v>1090</v>
+      </c>
+      <c r="S11">
+        <v>0</v>
+      </c>
+      <c r="T11">
+        <v>1090</v>
+      </c>
+      <c r="U11">
+        <v>1090</v>
+      </c>
+      <c r="V11">
+        <v>1090</v>
+      </c>
+      <c r="W11">
+        <v>1090</v>
+      </c>
+      <c r="X11">
+        <v>1090</v>
+      </c>
+      <c r="Y11">
+        <v>785</v>
+      </c>
+      <c r="Z11">
+        <v>0</v>
+      </c>
+      <c r="AA11">
+        <v>0</v>
+      </c>
+      <c r="AB11">
+        <v>0</v>
+      </c>
+      <c r="AC11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
         <v>63</v>
       </c>
-    </row>
-    <row r="21" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="F20">
+        <v>2.5000000000000001E-4</v>
+      </c>
+      <c r="G20">
+        <v>512</v>
+      </c>
+      <c r="H20">
+        <v>3</v>
+      </c>
+      <c r="I20">
+        <v>0.3</v>
+      </c>
+      <c r="J20">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="21" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C21" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="22" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C22" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="23" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C23" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C24" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="25" spans="3:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C25" t="s">
         <v>68</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F11">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G11">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H2:H11">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="R2:R11">
+    <cfRule type="colorScale" priority="16">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S2:S11">
     <cfRule type="colorScale" priority="15">
       <colorScale>
         <cfvo type="min"/>
@@ -2655,31 +2891,43 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G11">
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H11">
-    <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R2:R11">
+  <conditionalFormatting sqref="T2:T11">
+    <cfRule type="colorScale" priority="14">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="U2:U11">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="V2:V11">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W2:W11">
     <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
@@ -2691,7 +2939,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S11">
+  <conditionalFormatting sqref="X2:X11">
     <cfRule type="colorScale" priority="10">
       <colorScale>
         <cfvo type="min"/>
@@ -2703,7 +2951,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="T2:T11">
+  <conditionalFormatting sqref="Y2:Y11">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -2715,7 +2963,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U2:U11">
+  <conditionalFormatting sqref="Z2:Z11">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -2727,7 +2975,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V2:V11">
+  <conditionalFormatting sqref="I2:I11">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -2739,7 +2987,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W2:W11">
+  <conditionalFormatting sqref="J2:J11">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -2751,7 +2999,31 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="X2:X11">
+  <conditionalFormatting sqref="F20">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G20">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H20">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -2763,31 +3035,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="Y2:Y11">
-    <cfRule type="colorScale" priority="4">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Z2:Z11">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I11">
+  <conditionalFormatting sqref="I20">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -2799,7 +3047,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J11">
+  <conditionalFormatting sqref="J20">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>

<commit_message>
feat: Implement stateful training resumption
</commit_message>
<xml_diff>
--- a/Eval_Run_Logs.xlsx
+++ b/Eval_Run_Logs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29119"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29204"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\DeepRL-MsPacman\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BC7E1B2-D1CE-40BE-93DA-2F190D5FC3EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF4D4A46-38C5-41FE-80F4-2CB8E297AF20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{0D67D52D-1513-48BB-A273-B9082DA3F499}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{0D67D52D-1513-48BB-A273-B9082DA3F499}"/>
   </bookViews>
   <sheets>
     <sheet name="DQN_Runs" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="78">
   <si>
     <t>Run ID</t>
   </si>
@@ -259,6 +259,18 @@
   </si>
   <si>
     <t>PPO Baseline - 10M steps - Optimal</t>
+  </si>
+  <si>
+    <t>Final</t>
+  </si>
+  <si>
+    <t>20-30 million</t>
+  </si>
+  <si>
+    <t>0-13 million</t>
+  </si>
+  <si>
+    <t>13-20 million</t>
   </si>
 </sst>
 </file>
@@ -1661,7 +1673,7 @@
         <v>500000</v>
       </c>
       <c r="H20">
-        <v>1000000</v>
+        <v>2500000</v>
       </c>
       <c r="I20">
         <v>10000</v>
@@ -1685,6 +1697,18 @@
   </sheetData>
   <conditionalFormatting sqref="F2:F12">
     <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G2:G12">
+    <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1827,25 +1851,13 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G12">
-    <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{606356CF-33ED-426F-8480-D5D1647FF48E}">
-  <dimension ref="A1:AC25"/>
+  <dimension ref="A1:AC27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
@@ -2903,7 +2915,10 @@
     </row>
     <row r="20" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
-        <v>63</v>
+        <v>74</v>
+      </c>
+      <c r="E20" t="s">
+        <v>76</v>
       </c>
       <c r="F20">
         <v>2.5000000000000001E-4</v>
@@ -2922,33 +2937,88 @@
       </c>
     </row>
     <row r="21" spans="3:10" x14ac:dyDescent="0.25">
-      <c r="C21" t="s">
-        <v>64</v>
+      <c r="E21" t="s">
+        <v>77</v>
+      </c>
+      <c r="F21">
+        <v>1E-4</v>
+      </c>
+      <c r="G21">
+        <v>1024</v>
+      </c>
+      <c r="H21">
+        <v>10</v>
+      </c>
+      <c r="I21">
+        <v>0.1</v>
+      </c>
+      <c r="J21">
+        <v>0.01</v>
       </c>
     </row>
     <row r="22" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C22" t="s">
-        <v>65</v>
+        <v>63</v>
+      </c>
+      <c r="E22" t="s">
+        <v>75</v>
+      </c>
+      <c r="F22">
+        <v>1E-4</v>
+      </c>
+      <c r="G22">
+        <v>1024</v>
+      </c>
+      <c r="H22">
+        <v>10</v>
+      </c>
+      <c r="I22">
+        <v>0.1</v>
+      </c>
+      <c r="J22">
+        <v>0.01</v>
       </c>
     </row>
     <row r="23" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C23" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="24" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C24" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="25" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C25" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C26" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="27" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C27" t="s">
         <v>68</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="F2:F12">
     <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F20">
+    <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -2971,8 +3041,80 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G20">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="H2:H12">
     <cfRule type="colorScale" priority="29">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H20">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I2:I12">
+    <cfRule type="colorScale" priority="12">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I20">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J2:J12">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="FFF8696B"/>
+        <color rgb="FFFFEB84"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J20">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -3091,90 +3233,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I12">
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J12">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F20">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G20">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H20">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I20">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J20">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFFEB84"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(evaluate): Add evaluations script and RAM-based reward wrapper
</commit_message>
<xml_diff>
--- a/Eval_Run_Logs.xlsx
+++ b/Eval_Run_Logs.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Github\DeepRL-MsPacman\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF4D4A46-38C5-41FE-80F4-2CB8E297AF20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{8A1E37F1-33CB-47C0-9960-B026AA7FDFE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{0D67D52D-1513-48BB-A273-B9082DA3F499}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{0D67D52D-1513-48BB-A273-B9082DA3F499}"/>
   </bookViews>
   <sheets>
     <sheet name="DQN_Runs" sheetId="1" r:id="rId1"/>
     <sheet name="PPO_Runs" sheetId="2" r:id="rId2"/>
+    <sheet name="Human" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="92">
   <si>
     <t>Run ID</t>
   </si>
@@ -271,16 +273,59 @@
   </si>
   <si>
     <t>13-20 million</t>
+  </si>
+  <si>
+    <t>Level 3</t>
+  </si>
+  <si>
+    <t>30-40 million</t>
+  </si>
+  <si>
+    <t>40-50 million</t>
+  </si>
+  <si>
+    <t>Level 4</t>
+  </si>
+  <si>
+    <t>timestep</t>
+  </si>
+  <si>
+    <t>run_name</t>
+  </si>
+  <si>
+    <t>agent_type</t>
+  </si>
+  <si>
+    <t>DQN_Run_12</t>
+  </si>
+  <si>
+    <t>dqn</t>
+  </si>
+  <si>
+    <t>PPO_Run_12</t>
+  </si>
+  <si>
+    <t>ppo</t>
+  </si>
+  <si>
+    <t>50-60 million</t>
+  </si>
+  <si>
+    <t>0-10 million</t>
+  </si>
+  <si>
+    <t>10-30 million</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.000000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -319,7 +364,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -328,6 +373,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -663,7 +709,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7BDCA7AB-C83E-496B-A323-D25B7B27B0B8}">
-  <dimension ref="A1:AA23"/>
+  <dimension ref="A1:AD48"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.7109375" bestFit="1" customWidth="1"/>
@@ -1497,6 +1543,15 @@
       <c r="X10">
         <v>136.22434043096499</v>
       </c>
+      <c r="Y10">
+        <v>0</v>
+      </c>
+      <c r="Z10">
+        <v>0</v>
+      </c>
+      <c r="AA10">
+        <v>0</v>
+      </c>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11">
@@ -1568,6 +1623,15 @@
       <c r="X11">
         <v>125.895688857664</v>
       </c>
+      <c r="Y11">
+        <v>0</v>
+      </c>
+      <c r="Z11">
+        <v>0</v>
+      </c>
+      <c r="AA11">
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12">
@@ -1649,7 +1713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:30" x14ac:dyDescent="0.25">
       <c r="B17" t="s">
         <v>60</v>
       </c>
@@ -1657,15 +1721,113 @@
         <v>61</v>
       </c>
     </row>
-    <row r="18" spans="2:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:30" ht="45" x14ac:dyDescent="0.25">
       <c r="C18" s="5" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="P18" t="s">
+        <v>46</v>
+      </c>
+      <c r="Q18" t="s">
+        <v>47</v>
+      </c>
+      <c r="R18" t="s">
+        <v>48</v>
+      </c>
+      <c r="S18" t="s">
+        <v>49</v>
+      </c>
+      <c r="T18" t="s">
+        <v>50</v>
+      </c>
+      <c r="U18" t="s">
+        <v>51</v>
+      </c>
+      <c r="V18" t="s">
+        <v>52</v>
+      </c>
+      <c r="W18" t="s">
+        <v>53</v>
+      </c>
+      <c r="X18" t="s">
+        <v>54</v>
+      </c>
+      <c r="Y18" t="s">
+        <v>55</v>
+      </c>
+      <c r="Z18" t="s">
+        <v>56</v>
+      </c>
+      <c r="AA18" t="s">
+        <v>57</v>
+      </c>
+      <c r="AB18" t="s">
+        <v>82</v>
+      </c>
+      <c r="AC18" t="s">
+        <v>83</v>
+      </c>
+      <c r="AD18" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="19" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="E19" t="s">
+        <v>63</v>
+      </c>
+      <c r="P19">
+        <v>675.7</v>
+      </c>
+      <c r="Q19">
+        <v>219.799058830164</v>
+      </c>
+      <c r="R19">
+        <v>350</v>
+      </c>
+      <c r="S19">
+        <v>630</v>
+      </c>
+      <c r="T19">
+        <v>630</v>
+      </c>
+      <c r="U19">
+        <v>702.5</v>
+      </c>
+      <c r="V19">
+        <v>1480</v>
+      </c>
+      <c r="W19">
+        <v>765.66</v>
+      </c>
+      <c r="X19">
+        <v>121.500735334683</v>
+      </c>
+      <c r="Y19">
+        <v>0</v>
+      </c>
+      <c r="Z19">
+        <v>0</v>
+      </c>
+      <c r="AA19">
+        <v>0</v>
+      </c>
+      <c r="AB19">
+        <v>1000000</v>
+      </c>
+      <c r="AC19" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD19" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="20" spans="2:30" x14ac:dyDescent="0.25">
       <c r="C20" t="s">
         <v>63</v>
       </c>
+      <c r="E20" t="s">
+        <v>90</v>
+      </c>
       <c r="F20">
         <v>2.5000000000000001E-4</v>
       </c>
@@ -1678,20 +1840,1360 @@
       <c r="I20">
         <v>10000</v>
       </c>
-    </row>
-    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="P20">
+        <v>1218.5</v>
+      </c>
+      <c r="Q20">
+        <v>273.209044173471</v>
+      </c>
+      <c r="R20">
+        <v>910</v>
+      </c>
+      <c r="S20">
+        <v>1020</v>
+      </c>
+      <c r="T20">
+        <v>1160</v>
+      </c>
+      <c r="U20">
+        <v>1270</v>
+      </c>
+      <c r="V20">
+        <v>2380</v>
+      </c>
+      <c r="W20">
+        <v>916.4</v>
+      </c>
+      <c r="X20">
+        <v>126.294988983824</v>
+      </c>
+      <c r="Y20">
+        <v>0</v>
+      </c>
+      <c r="Z20">
+        <v>0</v>
+      </c>
+      <c r="AA20">
+        <v>0</v>
+      </c>
+      <c r="AB20">
+        <v>2000000</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD20" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="21" spans="2:30" x14ac:dyDescent="0.25">
       <c r="C21" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="E21" t="s">
+        <v>91</v>
+      </c>
+      <c r="F21">
+        <v>1E-4</v>
+      </c>
+      <c r="G21">
+        <v>500000</v>
+      </c>
+      <c r="H21">
+        <v>2500000</v>
+      </c>
+      <c r="I21">
+        <v>20000</v>
+      </c>
+      <c r="P21">
+        <v>1255.5</v>
+      </c>
+      <c r="Q21">
+        <v>320.22837494702401</v>
+      </c>
+      <c r="R21">
+        <v>850</v>
+      </c>
+      <c r="S21">
+        <v>1090</v>
+      </c>
+      <c r="T21">
+        <v>1150</v>
+      </c>
+      <c r="U21">
+        <v>1282.5</v>
+      </c>
+      <c r="V21">
+        <v>2660</v>
+      </c>
+      <c r="W21">
+        <v>786.52</v>
+      </c>
+      <c r="X21">
+        <v>103.11751460436599</v>
+      </c>
+      <c r="Y21">
+        <v>0</v>
+      </c>
+      <c r="Z21">
+        <v>0</v>
+      </c>
+      <c r="AA21">
+        <v>0</v>
+      </c>
+      <c r="AB21">
+        <v>3000000</v>
+      </c>
+      <c r="AC21" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD21" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="22" spans="2:30" x14ac:dyDescent="0.25">
       <c r="C22" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="P22">
+        <v>1051.7</v>
+      </c>
+      <c r="Q22">
+        <v>589.58649265670203</v>
+      </c>
+      <c r="R22">
+        <v>350</v>
+      </c>
+      <c r="S22">
+        <v>550</v>
+      </c>
+      <c r="T22">
+        <v>940</v>
+      </c>
+      <c r="U22">
+        <v>1385</v>
+      </c>
+      <c r="V22">
+        <v>2680</v>
+      </c>
+      <c r="W22">
+        <v>821.04</v>
+      </c>
+      <c r="X22">
+        <v>137.21058945498999</v>
+      </c>
+      <c r="Y22">
+        <v>0</v>
+      </c>
+      <c r="Z22">
+        <v>0</v>
+      </c>
+      <c r="AA22">
+        <v>0</v>
+      </c>
+      <c r="AB22">
+        <v>4000000</v>
+      </c>
+      <c r="AC22" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD22" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="23" spans="2:30" x14ac:dyDescent="0.25">
       <c r="C23" t="s">
         <v>71</v>
+      </c>
+      <c r="P23">
+        <v>2294</v>
+      </c>
+      <c r="Q23">
+        <v>1102.45364546725</v>
+      </c>
+      <c r="R23">
+        <v>340</v>
+      </c>
+      <c r="S23">
+        <v>1465</v>
+      </c>
+      <c r="T23">
+        <v>2330</v>
+      </c>
+      <c r="U23">
+        <v>2810</v>
+      </c>
+      <c r="V23">
+        <v>4470</v>
+      </c>
+      <c r="W23">
+        <v>794.88</v>
+      </c>
+      <c r="X23">
+        <v>119.80483118705</v>
+      </c>
+      <c r="Y23">
+        <v>0</v>
+      </c>
+      <c r="Z23">
+        <v>0</v>
+      </c>
+      <c r="AA23">
+        <v>0</v>
+      </c>
+      <c r="AB23">
+        <v>5000000</v>
+      </c>
+      <c r="AC23" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD23" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="24" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="P24">
+        <v>1506.9</v>
+      </c>
+      <c r="Q24">
+        <v>451.74788490390398</v>
+      </c>
+      <c r="R24">
+        <v>370</v>
+      </c>
+      <c r="S24">
+        <v>1310</v>
+      </c>
+      <c r="T24">
+        <v>1360</v>
+      </c>
+      <c r="U24">
+        <v>1470</v>
+      </c>
+      <c r="V24">
+        <v>3240</v>
+      </c>
+      <c r="W24">
+        <v>802.02</v>
+      </c>
+      <c r="X24">
+        <v>149.71933203109799</v>
+      </c>
+      <c r="Y24">
+        <v>0</v>
+      </c>
+      <c r="Z24">
+        <v>0</v>
+      </c>
+      <c r="AA24">
+        <v>0</v>
+      </c>
+      <c r="AB24">
+        <v>6000000</v>
+      </c>
+      <c r="AC24" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD24" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="25" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="P25">
+        <v>2550.4</v>
+      </c>
+      <c r="Q25">
+        <v>671.87799517772498</v>
+      </c>
+      <c r="R25">
+        <v>1010</v>
+      </c>
+      <c r="S25">
+        <v>1992.5</v>
+      </c>
+      <c r="T25">
+        <v>2520</v>
+      </c>
+      <c r="U25">
+        <v>2970</v>
+      </c>
+      <c r="V25">
+        <v>4400</v>
+      </c>
+      <c r="W25">
+        <v>880.54</v>
+      </c>
+      <c r="X25">
+        <v>114.53793161122501</v>
+      </c>
+      <c r="Y25">
+        <v>0</v>
+      </c>
+      <c r="Z25">
+        <v>0</v>
+      </c>
+      <c r="AA25">
+        <v>0</v>
+      </c>
+      <c r="AB25">
+        <v>7000000</v>
+      </c>
+      <c r="AC25" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD25" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="26" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="P26">
+        <v>2320.1999999999998</v>
+      </c>
+      <c r="Q26">
+        <v>893.74931517950699</v>
+      </c>
+      <c r="R26">
+        <v>790</v>
+      </c>
+      <c r="S26">
+        <v>1637.5</v>
+      </c>
+      <c r="T26">
+        <v>2225</v>
+      </c>
+      <c r="U26">
+        <v>2940</v>
+      </c>
+      <c r="V26">
+        <v>4770</v>
+      </c>
+      <c r="W26">
+        <v>790.7</v>
+      </c>
+      <c r="X26">
+        <v>137.414325926</v>
+      </c>
+      <c r="Y26">
+        <v>0</v>
+      </c>
+      <c r="Z26">
+        <v>0</v>
+      </c>
+      <c r="AA26">
+        <v>0</v>
+      </c>
+      <c r="AB26">
+        <v>8000000</v>
+      </c>
+      <c r="AC26" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD26" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="27" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="P27">
+        <v>2197.4</v>
+      </c>
+      <c r="Q27">
+        <v>612.26788221819902</v>
+      </c>
+      <c r="R27">
+        <v>1370</v>
+      </c>
+      <c r="S27">
+        <v>1740</v>
+      </c>
+      <c r="T27">
+        <v>2015</v>
+      </c>
+      <c r="U27">
+        <v>2535</v>
+      </c>
+      <c r="V27">
+        <v>4090</v>
+      </c>
+      <c r="W27">
+        <v>828.76</v>
+      </c>
+      <c r="X27">
+        <v>164.38468802344499</v>
+      </c>
+      <c r="Y27">
+        <v>0</v>
+      </c>
+      <c r="Z27">
+        <v>0</v>
+      </c>
+      <c r="AA27">
+        <v>0</v>
+      </c>
+      <c r="AB27">
+        <v>9000000</v>
+      </c>
+      <c r="AC27" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD27" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="28" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="P28">
+        <v>1994.5</v>
+      </c>
+      <c r="Q28">
+        <v>653.522506625951</v>
+      </c>
+      <c r="R28">
+        <v>840</v>
+      </c>
+      <c r="S28">
+        <v>1535</v>
+      </c>
+      <c r="T28">
+        <v>1800</v>
+      </c>
+      <c r="U28">
+        <v>2350</v>
+      </c>
+      <c r="V28">
+        <v>4380</v>
+      </c>
+      <c r="W28">
+        <v>779.2</v>
+      </c>
+      <c r="X28">
+        <v>114.766165428983</v>
+      </c>
+      <c r="Y28">
+        <v>0</v>
+      </c>
+      <c r="Z28">
+        <v>0</v>
+      </c>
+      <c r="AA28">
+        <v>0</v>
+      </c>
+      <c r="AB28">
+        <v>10000000</v>
+      </c>
+      <c r="AC28" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD28" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="29" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="P29">
+        <v>2507</v>
+      </c>
+      <c r="Q29">
+        <v>745.78478765321404</v>
+      </c>
+      <c r="R29">
+        <v>1440</v>
+      </c>
+      <c r="S29">
+        <v>2000</v>
+      </c>
+      <c r="T29">
+        <v>2345</v>
+      </c>
+      <c r="U29">
+        <v>2992.5</v>
+      </c>
+      <c r="V29">
+        <v>5750</v>
+      </c>
+      <c r="W29">
+        <v>903.8</v>
+      </c>
+      <c r="X29">
+        <v>121.62901036190399</v>
+      </c>
+      <c r="Y29">
+        <v>0</v>
+      </c>
+      <c r="Z29">
+        <v>0</v>
+      </c>
+      <c r="AA29">
+        <v>0</v>
+      </c>
+      <c r="AB29">
+        <v>11000000</v>
+      </c>
+      <c r="AC29" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD29" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="30" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="P30">
+        <v>1770.3</v>
+      </c>
+      <c r="Q30">
+        <v>536.28436411284497</v>
+      </c>
+      <c r="R30">
+        <v>1100</v>
+      </c>
+      <c r="S30">
+        <v>1387.5</v>
+      </c>
+      <c r="T30">
+        <v>1585</v>
+      </c>
+      <c r="U30">
+        <v>2062.5</v>
+      </c>
+      <c r="V30">
+        <v>5050</v>
+      </c>
+      <c r="W30">
+        <v>814.02</v>
+      </c>
+      <c r="X30">
+        <v>163.12639828728399</v>
+      </c>
+      <c r="Y30">
+        <v>0</v>
+      </c>
+      <c r="Z30">
+        <v>0</v>
+      </c>
+      <c r="AA30">
+        <v>0</v>
+      </c>
+      <c r="AB30">
+        <v>12000000</v>
+      </c>
+      <c r="AC30" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD30" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="31" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="P31">
+        <v>2494.1999999999998</v>
+      </c>
+      <c r="Q31">
+        <v>638.53395850308198</v>
+      </c>
+      <c r="R31">
+        <v>1210</v>
+      </c>
+      <c r="S31">
+        <v>2105</v>
+      </c>
+      <c r="T31">
+        <v>2445</v>
+      </c>
+      <c r="U31">
+        <v>2762.5</v>
+      </c>
+      <c r="V31">
+        <v>4340</v>
+      </c>
+      <c r="W31">
+        <v>860.24</v>
+      </c>
+      <c r="X31">
+        <v>124.718278086609</v>
+      </c>
+      <c r="Y31">
+        <v>0</v>
+      </c>
+      <c r="Z31">
+        <v>0</v>
+      </c>
+      <c r="AA31">
+        <v>0</v>
+      </c>
+      <c r="AB31">
+        <v>13000000</v>
+      </c>
+      <c r="AC31" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD31" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="32" spans="2:30" x14ac:dyDescent="0.25">
+      <c r="P32">
+        <v>2683.1</v>
+      </c>
+      <c r="Q32">
+        <v>665.613858089514</v>
+      </c>
+      <c r="R32">
+        <v>570</v>
+      </c>
+      <c r="S32">
+        <v>2337.5</v>
+      </c>
+      <c r="T32">
+        <v>2680</v>
+      </c>
+      <c r="U32">
+        <v>3122.5</v>
+      </c>
+      <c r="V32">
+        <v>4420</v>
+      </c>
+      <c r="W32">
+        <v>890.26</v>
+      </c>
+      <c r="X32">
+        <v>103.79764890975</v>
+      </c>
+      <c r="Y32">
+        <v>0</v>
+      </c>
+      <c r="Z32">
+        <v>0</v>
+      </c>
+      <c r="AA32">
+        <v>0</v>
+      </c>
+      <c r="AB32">
+        <v>14000000</v>
+      </c>
+      <c r="AC32" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD32" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="33" spans="16:30" x14ac:dyDescent="0.25">
+      <c r="P33">
+        <v>2951.9</v>
+      </c>
+      <c r="Q33">
+        <v>683.81977512242497</v>
+      </c>
+      <c r="R33">
+        <v>1780</v>
+      </c>
+      <c r="S33">
+        <v>2462.5</v>
+      </c>
+      <c r="T33">
+        <v>2660</v>
+      </c>
+      <c r="U33">
+        <v>3622.5</v>
+      </c>
+      <c r="V33">
+        <v>4390</v>
+      </c>
+      <c r="W33">
+        <v>873.94</v>
+      </c>
+      <c r="X33">
+        <v>137.92179162866299</v>
+      </c>
+      <c r="Y33">
+        <v>0</v>
+      </c>
+      <c r="Z33">
+        <v>0</v>
+      </c>
+      <c r="AA33">
+        <v>0</v>
+      </c>
+      <c r="AB33">
+        <v>15000000</v>
+      </c>
+      <c r="AC33" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD33" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="34" spans="16:30" x14ac:dyDescent="0.25">
+      <c r="P34">
+        <v>2649.6</v>
+      </c>
+      <c r="Q34">
+        <v>965.07802584018805</v>
+      </c>
+      <c r="R34">
+        <v>690</v>
+      </c>
+      <c r="S34">
+        <v>2220</v>
+      </c>
+      <c r="T34">
+        <v>2450</v>
+      </c>
+      <c r="U34">
+        <v>2630</v>
+      </c>
+      <c r="V34">
+        <v>7440</v>
+      </c>
+      <c r="W34">
+        <v>791.8</v>
+      </c>
+      <c r="X34">
+        <v>131.176802580919</v>
+      </c>
+      <c r="Y34">
+        <v>0</v>
+      </c>
+      <c r="Z34">
+        <v>0</v>
+      </c>
+      <c r="AA34">
+        <v>0</v>
+      </c>
+      <c r="AB34">
+        <v>16000000</v>
+      </c>
+      <c r="AC34" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD34" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="35" spans="16:30" x14ac:dyDescent="0.25">
+      <c r="P35">
+        <v>2227.8000000000002</v>
+      </c>
+      <c r="Q35">
+        <v>770.87066084887101</v>
+      </c>
+      <c r="R35">
+        <v>310</v>
+      </c>
+      <c r="S35">
+        <v>1690</v>
+      </c>
+      <c r="T35">
+        <v>2390</v>
+      </c>
+      <c r="U35">
+        <v>2675</v>
+      </c>
+      <c r="V35">
+        <v>4180</v>
+      </c>
+      <c r="W35">
+        <v>820.34</v>
+      </c>
+      <c r="X35">
+        <v>125.01476438057701</v>
+      </c>
+      <c r="Y35">
+        <v>0</v>
+      </c>
+      <c r="Z35">
+        <v>0</v>
+      </c>
+      <c r="AA35">
+        <v>0</v>
+      </c>
+      <c r="AB35">
+        <v>17000000</v>
+      </c>
+      <c r="AC35" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD35" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="36" spans="16:30" x14ac:dyDescent="0.25">
+      <c r="P36">
+        <v>2445.5</v>
+      </c>
+      <c r="Q36">
+        <v>630.47581038034002</v>
+      </c>
+      <c r="R36">
+        <v>720</v>
+      </c>
+      <c r="S36">
+        <v>2287.5</v>
+      </c>
+      <c r="T36">
+        <v>2370</v>
+      </c>
+      <c r="U36">
+        <v>2620</v>
+      </c>
+      <c r="V36">
+        <v>4120</v>
+      </c>
+      <c r="W36">
+        <v>861.92</v>
+      </c>
+      <c r="X36">
+        <v>117.631995922225</v>
+      </c>
+      <c r="Y36">
+        <v>0</v>
+      </c>
+      <c r="Z36">
+        <v>0</v>
+      </c>
+      <c r="AA36">
+        <v>0</v>
+      </c>
+      <c r="AB36">
+        <v>18000000</v>
+      </c>
+      <c r="AC36" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD36" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="37" spans="16:30" x14ac:dyDescent="0.25">
+      <c r="P37">
+        <v>2075.8000000000002</v>
+      </c>
+      <c r="Q37">
+        <v>573.06050591045198</v>
+      </c>
+      <c r="R37">
+        <v>250</v>
+      </c>
+      <c r="S37">
+        <v>2010</v>
+      </c>
+      <c r="T37">
+        <v>2310</v>
+      </c>
+      <c r="U37">
+        <v>2415</v>
+      </c>
+      <c r="V37">
+        <v>2880</v>
+      </c>
+      <c r="W37">
+        <v>728.82</v>
+      </c>
+      <c r="X37">
+        <v>135.90076444883499</v>
+      </c>
+      <c r="Y37">
+        <v>0</v>
+      </c>
+      <c r="Z37">
+        <v>0</v>
+      </c>
+      <c r="AA37">
+        <v>0</v>
+      </c>
+      <c r="AB37">
+        <v>19000000</v>
+      </c>
+      <c r="AC37" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD37" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="38" spans="16:30" x14ac:dyDescent="0.25">
+      <c r="P38">
+        <v>2051.1</v>
+      </c>
+      <c r="Q38">
+        <v>392.8062595934</v>
+      </c>
+      <c r="R38">
+        <v>1180</v>
+      </c>
+      <c r="S38">
+        <v>1940</v>
+      </c>
+      <c r="T38">
+        <v>2030</v>
+      </c>
+      <c r="U38">
+        <v>2270</v>
+      </c>
+      <c r="V38">
+        <v>3940</v>
+      </c>
+      <c r="W38">
+        <v>720.6</v>
+      </c>
+      <c r="X38">
+        <v>141.50846781958401</v>
+      </c>
+      <c r="Y38">
+        <v>0</v>
+      </c>
+      <c r="Z38">
+        <v>0</v>
+      </c>
+      <c r="AA38">
+        <v>0</v>
+      </c>
+      <c r="AB38">
+        <v>20000000</v>
+      </c>
+      <c r="AC38" t="s">
+        <v>85</v>
+      </c>
+      <c r="AD38" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="39" spans="16:30" x14ac:dyDescent="0.25">
+      <c r="P39">
+        <v>4098.2</v>
+      </c>
+      <c r="Q39">
+        <v>1156.0026737936901</v>
+      </c>
+      <c r="R39">
+        <v>1360</v>
+      </c>
+      <c r="S39">
+        <v>3167.5</v>
+      </c>
+      <c r="T39">
+        <v>4460</v>
+      </c>
+      <c r="U39">
+        <v>4790</v>
+      </c>
+      <c r="V39">
+        <v>6980</v>
+      </c>
+      <c r="W39">
+        <v>892.58</v>
+      </c>
+      <c r="X39">
+        <v>182.364114625192</v>
+      </c>
+      <c r="Y39">
+        <v>0</v>
+      </c>
+      <c r="Z39">
+        <v>0</v>
+      </c>
+      <c r="AA39">
+        <v>0</v>
+      </c>
+      <c r="AB39">
+        <v>21000000</v>
+      </c>
+      <c r="AC39" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="40" spans="16:30" x14ac:dyDescent="0.25">
+      <c r="P40">
+        <v>2739</v>
+      </c>
+      <c r="Q40">
+        <v>1159.9978230561201</v>
+      </c>
+      <c r="R40">
+        <v>730</v>
+      </c>
+      <c r="S40">
+        <v>2140</v>
+      </c>
+      <c r="T40">
+        <v>2625</v>
+      </c>
+      <c r="U40">
+        <v>3317.5</v>
+      </c>
+      <c r="V40">
+        <v>6110</v>
+      </c>
+      <c r="W40">
+        <v>824.48</v>
+      </c>
+      <c r="X40">
+        <v>111.32248903818299</v>
+      </c>
+      <c r="Y40">
+        <v>0</v>
+      </c>
+      <c r="Z40">
+        <v>0</v>
+      </c>
+      <c r="AA40">
+        <v>0</v>
+      </c>
+      <c r="AB40">
+        <v>22000000</v>
+      </c>
+      <c r="AC40" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="41" spans="16:30" x14ac:dyDescent="0.25">
+      <c r="P41">
+        <v>3699.9</v>
+      </c>
+      <c r="Q41">
+        <v>977.19604538245596</v>
+      </c>
+      <c r="R41">
+        <v>1210</v>
+      </c>
+      <c r="S41">
+        <v>3707.5</v>
+      </c>
+      <c r="T41">
+        <v>3800</v>
+      </c>
+      <c r="U41">
+        <v>4142.5</v>
+      </c>
+      <c r="V41">
+        <v>6160</v>
+      </c>
+      <c r="W41">
+        <v>809.14</v>
+      </c>
+      <c r="X41">
+        <v>120.619027930877</v>
+      </c>
+      <c r="Y41">
+        <v>0</v>
+      </c>
+      <c r="Z41">
+        <v>0</v>
+      </c>
+      <c r="AA41">
+        <v>0</v>
+      </c>
+      <c r="AB41">
+        <v>23000000</v>
+      </c>
+      <c r="AC41" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="42" spans="16:30" x14ac:dyDescent="0.25">
+      <c r="P42">
+        <v>3991</v>
+      </c>
+      <c r="Q42">
+        <v>940.71378444371896</v>
+      </c>
+      <c r="R42">
+        <v>2070</v>
+      </c>
+      <c r="S42">
+        <v>3687.5</v>
+      </c>
+      <c r="T42">
+        <v>4060</v>
+      </c>
+      <c r="U42">
+        <v>4447.5</v>
+      </c>
+      <c r="V42">
+        <v>6960</v>
+      </c>
+      <c r="W42">
+        <v>791.88</v>
+      </c>
+      <c r="X42">
+        <v>108.79368668551599</v>
+      </c>
+      <c r="Y42">
+        <v>0</v>
+      </c>
+      <c r="Z42">
+        <v>0</v>
+      </c>
+      <c r="AA42">
+        <v>0</v>
+      </c>
+      <c r="AB42">
+        <v>24000000</v>
+      </c>
+      <c r="AC42" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="43" spans="16:30" x14ac:dyDescent="0.25">
+      <c r="P43">
+        <v>3605.8</v>
+      </c>
+      <c r="Q43">
+        <v>1127.50119711464</v>
+      </c>
+      <c r="R43">
+        <v>760</v>
+      </c>
+      <c r="S43">
+        <v>2957.5</v>
+      </c>
+      <c r="T43">
+        <v>3890</v>
+      </c>
+      <c r="U43">
+        <v>4172.5</v>
+      </c>
+      <c r="V43">
+        <v>5790</v>
+      </c>
+      <c r="W43">
+        <v>814.74</v>
+      </c>
+      <c r="X43">
+        <v>194.39097435089599</v>
+      </c>
+      <c r="Y43">
+        <v>0</v>
+      </c>
+      <c r="Z43">
+        <v>0</v>
+      </c>
+      <c r="AA43">
+        <v>0</v>
+      </c>
+      <c r="AB43">
+        <v>25000000</v>
+      </c>
+      <c r="AC43" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="44" spans="16:30" x14ac:dyDescent="0.25">
+      <c r="P44">
+        <v>3784.2</v>
+      </c>
+      <c r="Q44">
+        <v>932.60163959850399</v>
+      </c>
+      <c r="R44">
+        <v>1370</v>
+      </c>
+      <c r="S44">
+        <v>3077.5</v>
+      </c>
+      <c r="T44">
+        <v>3880</v>
+      </c>
+      <c r="U44">
+        <v>4270</v>
+      </c>
+      <c r="V44">
+        <v>6960</v>
+      </c>
+      <c r="W44">
+        <v>823.66</v>
+      </c>
+      <c r="X44">
+        <v>157.800040967336</v>
+      </c>
+      <c r="Y44">
+        <v>0</v>
+      </c>
+      <c r="Z44">
+        <v>0</v>
+      </c>
+      <c r="AA44">
+        <v>0</v>
+      </c>
+      <c r="AB44">
+        <v>26000000</v>
+      </c>
+      <c r="AC44" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="45" spans="16:30" x14ac:dyDescent="0.25">
+      <c r="P45">
+        <v>3566.4</v>
+      </c>
+      <c r="Q45">
+        <v>965.52337824590904</v>
+      </c>
+      <c r="R45">
+        <v>1210</v>
+      </c>
+      <c r="S45">
+        <v>3787.5</v>
+      </c>
+      <c r="T45">
+        <v>3950</v>
+      </c>
+      <c r="U45">
+        <v>4055</v>
+      </c>
+      <c r="V45">
+        <v>4630</v>
+      </c>
+      <c r="W45">
+        <v>760.86</v>
+      </c>
+      <c r="X45">
+        <v>107.60055386437</v>
+      </c>
+      <c r="Y45">
+        <v>0</v>
+      </c>
+      <c r="Z45">
+        <v>0</v>
+      </c>
+      <c r="AA45">
+        <v>0</v>
+      </c>
+      <c r="AB45">
+        <v>27000000</v>
+      </c>
+      <c r="AC45" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="46" spans="16:30" x14ac:dyDescent="0.25">
+      <c r="P46">
+        <v>3795.4</v>
+      </c>
+      <c r="Q46">
+        <v>851.13758695007198</v>
+      </c>
+      <c r="R46">
+        <v>430</v>
+      </c>
+      <c r="S46">
+        <v>3890</v>
+      </c>
+      <c r="T46">
+        <v>3920</v>
+      </c>
+      <c r="U46">
+        <v>4150</v>
+      </c>
+      <c r="V46">
+        <v>5350</v>
+      </c>
+      <c r="W46">
+        <v>864.46</v>
+      </c>
+      <c r="X46">
+        <v>76.796388277869198</v>
+      </c>
+      <c r="Y46">
+        <v>0</v>
+      </c>
+      <c r="Z46">
+        <v>0</v>
+      </c>
+      <c r="AA46">
+        <v>0</v>
+      </c>
+      <c r="AB46">
+        <v>28000000</v>
+      </c>
+      <c r="AC46" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="47" spans="16:30" x14ac:dyDescent="0.25">
+      <c r="P47">
+        <v>4316.8</v>
+      </c>
+      <c r="Q47">
+        <v>1255.09618127154</v>
+      </c>
+      <c r="R47">
+        <v>930</v>
+      </c>
+      <c r="S47">
+        <v>4027.5</v>
+      </c>
+      <c r="T47">
+        <v>4520</v>
+      </c>
+      <c r="U47">
+        <v>4730</v>
+      </c>
+      <c r="V47">
+        <v>8320</v>
+      </c>
+      <c r="W47">
+        <v>899.74</v>
+      </c>
+      <c r="X47">
+        <v>93.083064892046593</v>
+      </c>
+      <c r="Y47">
+        <v>0</v>
+      </c>
+      <c r="Z47">
+        <v>0</v>
+      </c>
+      <c r="AA47">
+        <v>0</v>
+      </c>
+      <c r="AB47">
+        <v>29000000</v>
+      </c>
+      <c r="AC47" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="48" spans="16:30" x14ac:dyDescent="0.25">
+      <c r="P48">
+        <v>3103.5</v>
+      </c>
+      <c r="Q48">
+        <v>904.46968110622902</v>
+      </c>
+      <c r="R48">
+        <v>510</v>
+      </c>
+      <c r="S48">
+        <v>2365</v>
+      </c>
+      <c r="T48">
+        <v>3590</v>
+      </c>
+      <c r="U48">
+        <v>3630</v>
+      </c>
+      <c r="V48">
+        <v>4570</v>
+      </c>
+      <c r="W48">
+        <v>741.5</v>
+      </c>
+      <c r="X48">
+        <v>76.581177633128405</v>
+      </c>
+      <c r="Y48">
+        <v>0</v>
+      </c>
+      <c r="Z48">
+        <v>0</v>
+      </c>
+      <c r="AA48">
+        <v>0</v>
+      </c>
+      <c r="AB48">
+        <v>30000000</v>
+      </c>
+      <c r="AC48" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>
@@ -2920,7 +4422,7 @@
       <c r="E20" t="s">
         <v>76</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="6">
         <v>2.5000000000000001E-4</v>
       </c>
       <c r="G20">
@@ -2940,7 +4442,7 @@
       <c r="E21" t="s">
         <v>77</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="6">
         <v>1E-4</v>
       </c>
       <c r="G21">
@@ -2963,7 +4465,7 @@
       <c r="E22" t="s">
         <v>75</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="6">
         <v>1E-4</v>
       </c>
       <c r="G22">
@@ -2983,15 +4485,69 @@
       <c r="C23" t="s">
         <v>64</v>
       </c>
+      <c r="E23" t="s">
+        <v>79</v>
+      </c>
+      <c r="F23" s="6">
+        <v>1E-4</v>
+      </c>
+      <c r="G23">
+        <v>1024</v>
+      </c>
+      <c r="H23">
+        <v>10</v>
+      </c>
+      <c r="I23">
+        <v>0.1</v>
+      </c>
+      <c r="J23">
+        <v>0.01</v>
+      </c>
     </row>
     <row r="24" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C24" t="s">
         <v>65</v>
       </c>
+      <c r="E24" t="s">
+        <v>80</v>
+      </c>
+      <c r="F24" s="6">
+        <v>2.5000000000000001E-5</v>
+      </c>
+      <c r="G24">
+        <v>2048</v>
+      </c>
+      <c r="H24">
+        <v>10</v>
+      </c>
+      <c r="I24">
+        <v>0.1</v>
+      </c>
+      <c r="J24">
+        <v>0.01</v>
+      </c>
     </row>
     <row r="25" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C25" t="s">
         <v>66</v>
+      </c>
+      <c r="E25" t="s">
+        <v>89</v>
+      </c>
+      <c r="F25" s="6">
+        <v>2.5000000000000001E-5</v>
+      </c>
+      <c r="G25">
+        <v>2048</v>
+      </c>
+      <c r="H25">
+        <v>10</v>
+      </c>
+      <c r="I25">
+        <v>0.1</v>
+      </c>
+      <c r="J25">
+        <v>0.01</v>
       </c>
     </row>
     <row r="26" spans="3:10" x14ac:dyDescent="0.25">
@@ -3235,4 +4791,375 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BF58B94-E51C-4AC9-96D9-2A3F1FAD1D88}">
+  <dimension ref="A1:O25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1">
+        <v>13080</v>
+      </c>
+      <c r="B1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>14070</v>
+      </c>
+      <c r="B2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>18550</v>
+      </c>
+      <c r="B3" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>16520</v>
+      </c>
+      <c r="B4" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>46</v>
+      </c>
+      <c r="B16" t="s">
+        <v>47</v>
+      </c>
+      <c r="C16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" t="s">
+        <v>49</v>
+      </c>
+      <c r="E16" t="s">
+        <v>50</v>
+      </c>
+      <c r="F16" t="s">
+        <v>51</v>
+      </c>
+      <c r="G16" t="s">
+        <v>52</v>
+      </c>
+      <c r="H16" t="s">
+        <v>53</v>
+      </c>
+      <c r="I16" t="s">
+        <v>54</v>
+      </c>
+      <c r="J16" t="s">
+        <v>55</v>
+      </c>
+      <c r="K16" t="s">
+        <v>56</v>
+      </c>
+      <c r="L16" t="s">
+        <v>57</v>
+      </c>
+      <c r="M16" t="s">
+        <v>82</v>
+      </c>
+      <c r="N16" t="s">
+        <v>83</v>
+      </c>
+      <c r="O16" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17">
+        <v>3011.5</v>
+      </c>
+      <c r="B17">
+        <v>899.53116299999999</v>
+      </c>
+      <c r="C17">
+        <v>1170</v>
+      </c>
+      <c r="D17">
+        <v>2187.5</v>
+      </c>
+      <c r="E17">
+        <v>3590</v>
+      </c>
+      <c r="F17">
+        <v>3630</v>
+      </c>
+      <c r="G17">
+        <v>4200</v>
+      </c>
+      <c r="H17">
+        <v>716.6</v>
+      </c>
+      <c r="I17">
+        <v>72.860736130000006</v>
+      </c>
+      <c r="J17">
+        <v>0</v>
+      </c>
+      <c r="K17">
+        <v>0</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+      <c r="M17">
+        <v>30000000</v>
+      </c>
+      <c r="N17" t="s">
+        <v>85</v>
+      </c>
+      <c r="O17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>322.7</v>
+      </c>
+      <c r="B18">
+        <v>72.583702990000006</v>
+      </c>
+      <c r="C18">
+        <v>310</v>
+      </c>
+      <c r="D18">
+        <v>310</v>
+      </c>
+      <c r="E18">
+        <v>310</v>
+      </c>
+      <c r="F18">
+        <v>310</v>
+      </c>
+      <c r="G18">
+        <v>740</v>
+      </c>
+      <c r="H18">
+        <v>557.98</v>
+      </c>
+      <c r="I18">
+        <v>28.460136930000001</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>0</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <v>30000000</v>
+      </c>
+      <c r="N18" t="s">
+        <v>87</v>
+      </c>
+      <c r="O18" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>3227.4</v>
+      </c>
+      <c r="B19">
+        <v>693.15356059999999</v>
+      </c>
+      <c r="C19">
+        <v>1110</v>
+      </c>
+      <c r="D19">
+        <v>3550</v>
+      </c>
+      <c r="E19">
+        <v>3550</v>
+      </c>
+      <c r="F19">
+        <v>3550</v>
+      </c>
+      <c r="G19">
+        <v>3550</v>
+      </c>
+      <c r="H19">
+        <v>712.02</v>
+      </c>
+      <c r="I19">
+        <v>97.383754060000001</v>
+      </c>
+      <c r="J19">
+        <v>0</v>
+      </c>
+      <c r="K19">
+        <v>0</v>
+      </c>
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19">
+        <v>60000000</v>
+      </c>
+      <c r="N19" t="s">
+        <v>87</v>
+      </c>
+      <c r="O19" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>46</v>
+      </c>
+      <c r="B23" t="s">
+        <v>47</v>
+      </c>
+      <c r="C23" t="s">
+        <v>48</v>
+      </c>
+      <c r="D23" t="s">
+        <v>49</v>
+      </c>
+      <c r="E23" t="s">
+        <v>50</v>
+      </c>
+      <c r="F23" t="s">
+        <v>51</v>
+      </c>
+      <c r="G23" t="s">
+        <v>52</v>
+      </c>
+      <c r="H23" t="s">
+        <v>53</v>
+      </c>
+      <c r="I23" t="s">
+        <v>54</v>
+      </c>
+      <c r="J23" t="s">
+        <v>55</v>
+      </c>
+      <c r="K23" t="s">
+        <v>56</v>
+      </c>
+      <c r="L23" t="s">
+        <v>57</v>
+      </c>
+      <c r="M23" t="s">
+        <v>82</v>
+      </c>
+      <c r="N23" t="s">
+        <v>83</v>
+      </c>
+      <c r="O23" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" s="4">
+        <v>3197.84</v>
+      </c>
+      <c r="B24" s="4">
+        <v>771.28405439999995</v>
+      </c>
+      <c r="C24" s="4">
+        <v>700</v>
+      </c>
+      <c r="D24" s="4">
+        <v>2977.5</v>
+      </c>
+      <c r="E24" s="4">
+        <v>3600</v>
+      </c>
+      <c r="F24" s="4">
+        <v>3630</v>
+      </c>
+      <c r="G24" s="4">
+        <v>5410</v>
+      </c>
+      <c r="H24" s="4">
+        <v>737.05600000000004</v>
+      </c>
+      <c r="I24" s="4">
+        <v>74.02028688</v>
+      </c>
+      <c r="J24">
+        <v>0</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+      <c r="L24">
+        <v>0</v>
+      </c>
+      <c r="M24">
+        <v>30000000</v>
+      </c>
+      <c r="N24" t="s">
+        <v>85</v>
+      </c>
+      <c r="O24" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" s="4">
+        <v>3160.26</v>
+      </c>
+      <c r="B25" s="4">
+        <v>719.85896279999997</v>
+      </c>
+      <c r="C25" s="4">
+        <v>530</v>
+      </c>
+      <c r="D25" s="4">
+        <v>3550</v>
+      </c>
+      <c r="E25" s="4">
+        <v>3550</v>
+      </c>
+      <c r="F25" s="4">
+        <v>3550</v>
+      </c>
+      <c r="G25" s="4">
+        <v>3550</v>
+      </c>
+      <c r="H25" s="4">
+        <v>707.36800000000005</v>
+      </c>
+      <c r="I25" s="4">
+        <v>83.860704810000001</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>0</v>
+      </c>
+      <c r="L25">
+        <v>0</v>
+      </c>
+      <c r="M25">
+        <v>60000000</v>
+      </c>
+      <c r="N25" t="s">
+        <v>87</v>
+      </c>
+      <c r="O25" t="s">
+        <v>88</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>